<commit_message>
Auto-select better subject rent source (CoStar vs RealPage) per market
- Add --realpage-subject-rents (RealPage per-property 10-yr export) as an
  alternative subject rent source. The script now picks whichever of CoStar /
  RealPage tracks HelloData more closely in the overlap, per deal/market, and
  level-aligns it. The chosen source shows in the row label and per-year detail.
- For Aura Beacon Island (Houston), RealPage wins (avg miss ~$87 vs CoStar ~$160)
  and correctly shows no pre-2022 history (the property was built in 2022, where
  CoStar was backfilling spurious rents). For Bella Mirage (Phoenix), CoStar wins.
- Subject occupancy fallback still comes from CoStar (RealPage 10-yr has none).
- Add the Houston RealPage rent file to the Aura example; update SKILL.md.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -2153,20 +2153,14 @@
     <row r="23" ht="14.4" customHeight="1">
       <c r="B23" s="28" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Market Rent  (CoStar→HD)</t>
-        </is>
-      </c>
-      <c r="C23" s="45" t="n">
-        <v>1529</v>
-      </c>
-      <c r="D23" s="45" t="n">
-        <v>1570</v>
-      </c>
-      <c r="E23" s="45" t="n">
-        <v>1636</v>
-      </c>
+          <t xml:space="preserve">  Market Rent  (RealPage→HD)</t>
+        </is>
+      </c>
+      <c r="C23" s="45" t="n"/>
+      <c r="D23" s="45" t="n"/>
+      <c r="E23" s="45" t="n"/>
       <c r="F23" s="45" t="n">
-        <v>1732</v>
+        <v>1795</v>
       </c>
       <c r="G23" s="45" t="n">
         <v>1854</v>
@@ -2228,17 +2222,11 @@
           <t xml:space="preserve">  Effective Rent</t>
         </is>
       </c>
-      <c r="C25" s="45" t="n">
-        <v>1502</v>
-      </c>
-      <c r="D25" s="45" t="n">
-        <v>1533</v>
-      </c>
-      <c r="E25" s="45" t="n">
-        <v>1636</v>
-      </c>
+      <c r="C25" s="45" t="n"/>
+      <c r="D25" s="45" t="n"/>
+      <c r="E25" s="45" t="n"/>
       <c r="F25" s="45" t="n">
-        <v>1675</v>
+        <v>1657</v>
       </c>
       <c r="G25" s="45" t="n">
         <v>1728</v>
@@ -2328,15 +2316,9 @@
           <t xml:space="preserve">  Concession %</t>
         </is>
       </c>
-      <c r="C28" s="50" t="n">
-        <v>0.01751046569192205</v>
-      </c>
-      <c r="D28" s="50" t="n">
-        <v>0.02358069974400357</v>
-      </c>
-      <c r="E28" s="50" t="n">
-        <v>6.844915329753041e-06</v>
-      </c>
+      <c r="C28" s="50" t="n"/>
+      <c r="D28" s="50" t="n"/>
+      <c r="E28" s="50" t="n"/>
       <c r="F28" s="50" t="n">
         <v>0.115411309062742</v>
       </c>
@@ -2903,7 +2885,7 @@
       </c>
       <c r="E52" s="57" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2897,7 @@
       </c>
       <c r="E53" s="57" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2909,7 @@
       </c>
       <c r="E54" s="57" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2921,7 @@
       </c>
       <c r="E55" s="57" t="inlineStr">
         <is>
-          <t>CoStar</t>
+          <t>RealPage</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make subject Concession % a live calculation
Concession % is now =(Market Rent − Effective Rent)/Market Rent per column
(IFERROR-guarded), derived from the displayed subject rent rows, matching the
hand-tweaked Bella Mirage version — instead of a static value.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -2319,17 +2319,21 @@
       <c r="C28" s="50" t="n"/>
       <c r="D28" s="50" t="n"/>
       <c r="E28" s="50" t="n"/>
-      <c r="F28" s="50" t="n">
-        <v>0.115411309062742</v>
-      </c>
-      <c r="G28" s="50" t="n">
-        <v>0.1190795285268549</v>
-      </c>
-      <c r="H28" s="50" t="n">
-        <v>0.07751519672607349</v>
-      </c>
-      <c r="I28" s="50" t="n">
-        <v>0.1335660919588936</v>
+      <c r="F28" s="50">
+        <f>IFERROR((F23-F25)/F23,"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="50">
+        <f>IFERROR((G23-G25)/G23,"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="50">
+        <f>IFERROR((H23-H25)/H23,"")</f>
+        <v/>
+      </c>
+      <c r="I28" s="50">
+        <f>IFERROR((I23-I25)/I23,"")</f>
+        <v/>
       </c>
       <c r="J28" s="51" t="n"/>
       <c r="K28" s="51" t="n"/>

</xml_diff>

<commit_message>
Diligence corrects buckets; map applies diligence; add Aura research example
- apply_diligence now corrects the auto-classification from researched status
  (e.g. a "proposed/permitted/stalled" deal CoStar called UC moves to PROPOSED).
- build_map takes --diligence: applies the same corrections so map buckets match
  the chart, and plots type=shadow rows.
- Add examples/aura_beacon_island/diligence.csv (real researched findings):
  confirmed UC drops 5->3 deals; Riverview & The League I -> Proposed; "Lenox
  Clear Creek" flagged as the OHT/Crow JV in Clear Lake; 4 proposed deals
  unverified; shadow supply thin/corridor-based.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Competitive Analysis" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Supply &amp; Absorption" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Reconciliation Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Diligence" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;;&quot;—&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +99,12 @@
       <name val="Calibri"/>
       <color rgb="FF000000"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="12">
@@ -184,7 +191,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -344,6 +351,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1004,7 +1015,7 @@
       <c r="B12" s="12" t="n"/>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION (5 properties, 1,486 units)</t>
+          <t>UNDER CONSTRUCTION (3 properties, 885 units)</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1033,7 @@
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q1 2027</t>
         </is>
       </c>
       <c r="F13" s="17" t="n"/>
@@ -1042,7 +1053,11 @@
           <t>Garden</t>
         </is>
       </c>
-      <c r="K13" s="15" t="n"/>
+      <c r="K13" s="15" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="14" t="n">
@@ -1058,7 +1073,7 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Q4 2027</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="F14" s="17" t="n"/>
@@ -1078,7 +1093,11 @@
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K14" s="15" t="n"/>
+      <c r="K14" s="15" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="B15" s="14" t="n">
@@ -1114,85 +1133,97 @@
           <t>Townhome</t>
         </is>
       </c>
-      <c r="K15" s="15" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="14" t="n">
+      <c r="K15" s="15" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>PROPOSED (7 properties, 1,963 units)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="21" t="n">
         <v>9</v>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>The League I</t>
         </is>
       </c>
-      <c r="D16" s="16" t="n">
+      <c r="D18" s="23" t="n">
         <v>304</v>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="n"/>
+      <c r="G18" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>MOS R.E LLC</t>
+        </is>
+      </c>
+      <c r="I18" s="21" t="n"/>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>Mid-Rise</t>
+        </is>
+      </c>
+      <c r="K18" s="22" t="inlineStr">
+        <is>
+          <t>Diligence: proposed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Riverview at Clear Creek</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>298</v>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
       </c>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="F19" s="24" t="n"/>
+      <c r="G19" s="25" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>MOS R.E LLC</t>
-        </is>
-      </c>
-      <c r="I16" s="14" t="n"/>
-      <c r="J16" s="14" t="inlineStr">
+      <c r="H19" s="22" t="inlineStr">
+        <is>
+          <t>Atticus Real Estate</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="n"/>
+      <c r="J19" s="21" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K16" s="15" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
-        <is>
-          <t>Riverview at Clear Creek</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="n">
-        <v>297</v>
-      </c>
-      <c r="E17" s="14" t="inlineStr">
-        <is>
-          <t>Q2 2028</t>
-        </is>
-      </c>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="inlineStr">
-        <is>
-          <t>Atticus Real Estate</t>
-        </is>
-      </c>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="14" t="inlineStr">
-        <is>
-          <t>Mid-Rise</t>
-        </is>
-      </c>
-      <c r="K17" s="15" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="20" t="inlineStr">
-        <is>
-          <t>PROPOSED (5 properties, 1,361 units)</t>
+      <c r="K19" s="22" t="inlineStr">
+        <is>
+          <t>Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1263,7 @@
       </c>
       <c r="K20" s="22" t="inlineStr">
         <is>
-          <t>Units: CoStar 260 vs RealPage 76</t>
+          <t>Units: CoStar 260 vs RealPage 76; Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1303,7 @@
       </c>
       <c r="K21" s="22" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1343,7 @@
       </c>
       <c r="K22" s="22" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1383,7 @@
       </c>
       <c r="K23" s="22" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1423,7 @@
       </c>
       <c r="K24" s="22" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -1406,10 +1437,10 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C5:K5"/>
-    <mergeCell ref="C19:K19"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="B27:K27"/>
     <mergeCell ref="B3:F3"/>
+    <mergeCell ref="C17:K17"/>
     <mergeCell ref="C12:K12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1578,15 +1609,15 @@
         </is>
       </c>
       <c r="R7" s="32">
-        <f>'Competitive Analysis'!C16</f>
+        <f>'Competitive Analysis'!C13</f>
         <v/>
       </c>
       <c r="S7" s="33">
-        <f>'Competitive Analysis'!D16</f>
+        <f>'Competitive Analysis'!D13</f>
         <v/>
       </c>
       <c r="T7" s="34">
-        <f>'Competitive Analysis'!E16</f>
+        <f>'Competitive Analysis'!E13</f>
         <v/>
       </c>
       <c r="V7">
@@ -1607,26 +1638,6 @@
       <c r="C8" s="36" t="n">
         <v>150</v>
       </c>
-      <c r="R8" s="32">
-        <f>'Competitive Analysis'!C17</f>
-        <v/>
-      </c>
-      <c r="S8" s="33">
-        <f>'Competitive Analysis'!D17</f>
-        <v/>
-      </c>
-      <c r="T8" s="34">
-        <f>'Competitive Analysis'!E17</f>
-        <v/>
-      </c>
-      <c r="V8">
-        <f>IFERROR(VALUE(RIGHT(T8,4))*4+MATCH(LEFT(T8,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W8">
-        <f>IF(V8="","",IF(V8&lt;=$Z$1,0,MAX(1,INT((V8-$Z$2)/4)+1)))</f>
-        <v/>
-      </c>
     </row>
     <row r="9" ht="14.4" customHeight="1">
       <c r="B9" s="28" t="inlineStr">
@@ -1637,25 +1648,10 @@
       <c r="C9" s="36" t="n">
         <v>325</v>
       </c>
-      <c r="R9" s="32">
-        <f>'Competitive Analysis'!C13</f>
-        <v/>
-      </c>
-      <c r="S9" s="33">
-        <f>'Competitive Analysis'!D13</f>
-        <v/>
-      </c>
-      <c r="T9" s="34">
-        <f>'Competitive Analysis'!E13</f>
-        <v/>
-      </c>
-      <c r="V9">
-        <f>IFERROR(VALUE(RIGHT(T9,4))*4+MATCH(LEFT(T9,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
-        <v/>
-      </c>
-      <c r="W9">
-        <f>IF(V9="","",IF(V9&lt;=$Z$1,0,MAX(1,INT((V9-$Z$2)/4)+1)))</f>
-        <v/>
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>PROPOSED PIPELINE (scenario toggle)</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="14.4" customHeight="1">
@@ -1667,6 +1663,26 @@
       <c r="C10" s="36" t="n">
         <v>500</v>
       </c>
+      <c r="R10" s="30" t="inlineStr">
+        <is>
+          <t>Property</t>
+        </is>
+      </c>
+      <c r="S10" s="30" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="T10" s="30" t="inlineStr">
+        <is>
+          <t>Est. Delivery</t>
+        </is>
+      </c>
+      <c r="U10" s="30" t="inlineStr">
+        <is>
+          <t>Built In</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="14.4" customHeight="1">
       <c r="B11" s="28" t="inlineStr">
@@ -1678,44 +1694,79 @@
         <f>IF($C$7="Bear",$C$8,IF($C$7="Bull",$C$10,$C$9))</f>
         <v/>
       </c>
-      <c r="R11" s="27" t="inlineStr">
-        <is>
-          <t>PROPOSED PIPELINE (scenario toggle)</t>
-        </is>
+      <c r="R11" s="32" t="inlineStr">
+        <is>
+          <t>The League Future Phases</t>
+        </is>
+      </c>
+      <c r="S11" s="33" t="n">
+        <v>400</v>
+      </c>
+      <c r="T11" s="38" t="inlineStr"/>
+      <c r="U11" s="38" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V11">
+        <f>IFERROR(VALUE(RIGHT(T11,4))*4+MATCH(LEFT(T11,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W11">
+        <f>IF(V11="","",IF(V11&lt;=$Z$1,0,MAX(1,INT((V11-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X11">
+        <f>IF(U11="All",1,IF(U11="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U11="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="14.4" customHeight="1">
-      <c r="R12" s="30" t="inlineStr">
-        <is>
-          <t>Property</t>
-        </is>
-      </c>
-      <c r="S12" s="30" t="inlineStr">
-        <is>
-          <t>Units</t>
-        </is>
-      </c>
-      <c r="T12" s="30" t="inlineStr">
-        <is>
-          <t>Est. Delivery</t>
-        </is>
-      </c>
-      <c r="U12" s="30" t="inlineStr">
-        <is>
-          <t>Built In</t>
-        </is>
+      <c r="R12" s="32" t="inlineStr">
+        <is>
+          <t>The League I</t>
+        </is>
+      </c>
+      <c r="S12" s="33" t="n">
+        <v>304</v>
+      </c>
+      <c r="T12" s="38" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="U12" s="38" t="inlineStr">
+        <is>
+          <t>Bear only</t>
+        </is>
+      </c>
+      <c r="V12">
+        <f>IFERROR(VALUE(RIGHT(T12,4))*4+MATCH(LEFT(T12,2),{"Q1","Q2","Q3","Q4"},0)-1,"")</f>
+        <v/>
+      </c>
+      <c r="W12">
+        <f>IF(V12="","",IF(V12&lt;=$Z$1,0,MAX(1,INT((V12-$Z$2)/4)+1)))</f>
+        <v/>
+      </c>
+      <c r="X12">
+        <f>IF(U12="All",1,IF(U12="Bear+Base",IF($Z$3&gt;=2,1,0),IF(U12="Bear only",IF($Z$3&gt;=3,1,0),0)))</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="14.4" customHeight="1">
       <c r="R13" s="32" t="inlineStr">
         <is>
-          <t>The League Future Phases</t>
+          <t>Riverview at Clear Creek</t>
         </is>
       </c>
       <c r="S13" s="33" t="n">
-        <v>400</v>
-      </c>
-      <c r="T13" s="38" t="inlineStr"/>
+        <v>298</v>
+      </c>
+      <c r="T13" s="38" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
       <c r="U13" s="38" t="inlineStr">
         <is>
           <t>Bear only</t>
@@ -2015,27 +2066,27 @@
         <v>0</v>
       </c>
       <c r="J19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,1)+SUMIFS($S$13:$S$17,$W$13:$W$17,1,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,1)+SUMIFS($S$11:$S$17,$W$11:$W$17,1,$X$11:$X$17,1)</f>
         <v/>
       </c>
       <c r="K19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,2)+SUMIFS($S$13:$S$17,$W$13:$W$17,2,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,2)+SUMIFS($S$11:$S$17,$W$11:$W$17,2,$X$11:$X$17,1)</f>
         <v/>
       </c>
       <c r="L19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,3)+SUMIFS($S$13:$S$17,$W$13:$W$17,3,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,3)+SUMIFS($S$11:$S$17,$W$11:$W$17,3,$X$11:$X$17,1)</f>
         <v/>
       </c>
       <c r="M19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,4)+SUMIFS($S$13:$S$17,$W$13:$W$17,4,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,4)+SUMIFS($S$11:$S$17,$W$11:$W$17,4,$X$11:$X$17,1)</f>
         <v/>
       </c>
       <c r="N19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,5)+SUMIFS($S$13:$S$17,$W$13:$W$17,5,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,5)+SUMIFS($S$11:$S$17,$W$11:$W$17,5,$X$11:$X$17,1)</f>
         <v/>
       </c>
       <c r="O19" s="42">
-        <f>SUMIFS($S$5:$S$9,$W$5:$W$9,6)+SUMIFS($S$13:$S$17,$W$13:$W$17,6,$X$13:$X$17,1)</f>
+        <f>SUMIFS($S$5:$S$7,$W$5:$W$7,6)+SUMIFS($S$11:$S$17,$W$11:$W$17,6,$X$11:$X$17,1)</f>
         <v/>
       </c>
     </row>
@@ -2973,7 +3024,7 @@
       </c>
       <c r="E59" s="57" t="inlineStr">
         <is>
-          <t>1,486 / 336</t>
+          <t>885 / 336</t>
         </is>
       </c>
     </row>
@@ -2994,7 +3045,7 @@
     <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Bear,Base,Bull"</formula1>
     </dataValidation>
-    <dataValidation sqref="U13 U14 U15 U16 U17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U11 U12 U13 U14 U15 U16 U17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Bear only,Bear+Base,All,None"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3336,19 +3387,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Riverview at Clear Creek</t>
+          <t>The Edge at Seabrook Town Centre</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>301 N Wesley Dr</t>
+          <t>2101 Humble Dr</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>297</v>
+        <v>320</v>
       </c>
       <c r="D7" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3366,31 +3417,35 @@
       <c r="J7" s="60" t="n"/>
       <c r="K7" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr"/>
+          <t>RealPage</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>The Edge at Seabrook Town Centre</t>
+          <t>Lenox Clear Creek</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2101 Humble Dr</t>
+          <t>16200 State Highway 3</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>320</v>
+        <v>336</v>
       </c>
       <c r="D8" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Q2 2028</t>
+          <t>Q3 2027</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3404,31 +3459,35 @@
       <c r="J8" s="60" t="n"/>
       <c r="K8" t="inlineStr">
         <is>
-          <t>RealPage</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr"/>
+          <t>CoStar+RealPage</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>The League I</t>
+          <t>Dakota at Kemah</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E FM 518 &amp; Main St</t>
+          <t>2801 Lawrence Rd</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>304</v>
+        <v>229</v>
       </c>
       <c r="D9" t="n">
-        <v>2028</v>
+        <v>2027</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Q2 2028</t>
+          <t>Q1 2027</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3445,33 +3504,37 @@
           <t>RealPage</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Diligence: under construction</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Lenox Clear Creek</t>
+          <t>Seabrook Plaza</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>16200 State Highway 3</t>
+          <t>3101 Nasa Pky</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>336</v>
+        <v>260</v>
       </c>
       <c r="D10" t="n">
         <v>2027</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Q4 2027</t>
+          <t>Q3 2028</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="G10" s="59" t="n"/>
@@ -3483,33 +3546,37 @@
           <t>CoStar+RealPage</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Units: CoStar 260 vs RealPage 76; Diligence: proposed</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dakota at Kemah</t>
+          <t>Riverview at Clear Creek</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2801 Lawrence Rd</t>
+          <t>301 N Wesley Dr</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>229</v>
+        <v>298</v>
       </c>
       <c r="D11" t="n">
         <v>2027</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Q2 2027</t>
+          <t>Q2 2028</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>UNDER CONSTRUCTION</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="G11" s="59" t="n"/>
@@ -3518,31 +3585,35 @@
       <c r="J11" s="60" t="n"/>
       <c r="K11" t="inlineStr">
         <is>
-          <t>RealPage</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr"/>
+          <t>CoStar+RealPage</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Diligence: proposed</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Seabrook Plaza</t>
+          <t>The League I</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>3101 Nasa Pky</t>
+          <t>E FM 518 &amp; Main St</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>260</v>
+        <v>304</v>
       </c>
       <c r="D12" t="n">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Q3 2028</t>
+          <t>Q3 2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -3556,12 +3627,12 @@
       <c r="J12" s="60" t="n"/>
       <c r="K12" t="inlineStr">
         <is>
-          <t>CoStar+RealPage</t>
+          <t>RealPage</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Units: CoStar 260 vs RealPage 76</t>
+          <t>Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -3595,7 +3666,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3700,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -3663,7 +3734,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
@@ -3697,11 +3768,533 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>RealPage pipeline (not yet in CoStar)</t>
+          <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="61" t="inlineStr">
+        <is>
+          <t>PIPELINE DILIGENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>Property / Site</t>
+        </is>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D3" s="39" t="inlineStr">
+        <is>
+          <t>Est. Delivery</t>
+        </is>
+      </c>
+      <c r="E3" s="39" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F3" s="39" t="inlineStr">
+        <is>
+          <t>Leasing Pace</t>
+        </is>
+      </c>
+      <c r="G3" s="39" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H3" s="39" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>Riverview at Clear Creek</t>
+        </is>
+      </c>
+      <c r="C4" s="62" t="inlineStr">
+        <is>
+          <t>298</t>
+        </is>
+      </c>
+      <c r="D4" s="62" t="n"/>
+      <c r="E4" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="n"/>
+      <c r="G4" s="32" t="inlineStr">
+        <is>
+          <t>WB Property Group; waterfront mixed-use (marina/hotel/townhomes) incl senior-housing component; CoStar 'under construction' NOT corroborated, public record stalls ~2022-23; market-rate; full plan ~2029</t>
+        </is>
+      </c>
+      <c r="H4" s="32" t="inlineStr">
+        <is>
+          <t>https://communityimpact.com/houston/bay-area/development/2022/04/22/making-a-destination-league-city-developer-sign-agreement-to-build-riverview/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Lenox Clear Creek</t>
+        </is>
+      </c>
+      <c r="C5" s="62" t="inlineStr">
+        <is>
+          <t>336</t>
+        </is>
+      </c>
+      <c r="D5" s="62" t="inlineStr">
+        <is>
+          <t>Q3 2027</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="inlineStr">
+        <is>
+          <t>under construction</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="n"/>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>Likely CoStar placeholder = OHT Partners + Crow Holdings JV, 16200 SH-3; broke ground late 2025; market-rate; LOCATION is Clear Lake 77058 (~Webster), NOT League City - weaker overlap</t>
+        </is>
+      </c>
+      <c r="H5" s="32" t="inlineStr">
+        <is>
+          <t>https://rebusinessonline.com/oht-partners-crow-holdings-break-ground-on-336-unit-multifamily-project-in-metro-houston/</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Dakota at Kemah</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="D6" s="62" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="inlineStr">
+        <is>
+          <t>under construction</t>
+        </is>
+      </c>
+      <c r="F6" s="32" t="n"/>
+      <c r="G6" s="32" t="inlineStr">
+        <is>
+          <t>Dakota Enterprises; mgmt The Mathis Group; 2801 Lawrence Rd Kemah; 10 three-story bldgs; groundbreaking Dec 9 2025; TDLR completion Jan 15 2027; market-rate luxury</t>
+        </is>
+      </c>
+      <c r="H6" s="32" t="inlineStr">
+        <is>
+          <t>https://communityimpact.com/houston/bay-area/government/2025/12/03/the-dakota-at-kemah-to-have-groundbreaking-ceremony/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>The League I</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
+      <c r="D7" s="62" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>CJ Development (Johnny Vassallo); $125M 44-ac mixed-use FM-518; 304 Phase-1 count UNCONFIRMED (public sourcing ~600 total); no verified groundbreaking, prior multi-yr stall - field-verify vertical status</t>
+        </is>
+      </c>
+      <c r="H7" s="32" t="inlineStr">
+        <is>
+          <t>https://communityimpact.com/houston/bay-area/development/2026/03/31/new-modern-retail-dining-space-coming-to-league-city/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>The Edge at Seabrook Town Centre</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="D8" s="62" t="inlineStr">
+        <is>
+          <t>Q2 2028</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>under construction</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="n"/>
+      <c r="G8" s="32" t="inlineStr">
+        <is>
+          <t>HS Development Group; $85M 19.5-ac mixed-use; broke ground Jan 2026 after ~3-yr financing stall; 4-story garden + 28.5k sf retail; market-rate (rents $1.5k-$3.1k); buildout Q2 2028</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="inlineStr">
+        <is>
+          <t>https://therealdeal.com/texas/2026/01/16/hs-development-groups-seabrook-town-centre-breaks-ground/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>The League Future Phases</t>
+        </is>
+      </c>
+      <c r="C9" s="62" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="D9" s="62" t="n"/>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="n"/>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>CJ Development; future tranche of The League (FM-518); total project described up to ~600 units across phases so 400 future phase plausible but specific count NOT independently verified; market-rate</t>
+        </is>
+      </c>
+      <c r="H9" s="32" t="inlineStr">
+        <is>
+          <t>https://communityimpact.com/houston/bay-area/development/2022/01/27/45-acre-mixed-use-development-the-league-to-bring-retail-restaurants-homes-to-league-city/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Residences at Highland Center</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>275</t>
+        </is>
+      </c>
+      <c r="D10" s="62" t="n"/>
+      <c r="E10" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>UNVERIFIED - no public news, city agenda, or developer source found tying a ~275-unit MF project to Highland Center; possible CoStar/RealPage early-stage or speculative entry</t>
+        </is>
+      </c>
+      <c r="H10" s="32" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Seabrook Plaza</t>
+        </is>
+      </c>
+      <c r="C11" s="62" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="D11" s="62" t="n"/>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="n"/>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>UNVERIFIED - could not confirm a 260-unit 'Seabrook Plaza' MF project; may be alias/duplicate of The Edge at Seabrook Town Centre or speculative CoStar entry</t>
+        </is>
+      </c>
+      <c r="H11" s="32" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>Avalon at Kemah I</t>
+        </is>
+      </c>
+      <c r="C12" s="62" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="D12" s="62" t="n"/>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="n"/>
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>UNVERIFIED - no public record of an 'Avalon at Kemah' apartment project; Kemah's only verified active MF is The Dakota; possible CoStar placeholder/rename</t>
+        </is>
+      </c>
+      <c r="H12" s="32" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>Avalon at Kemah II</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="D13" s="62" t="n"/>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="n"/>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>UNVERIFIED - Phase II of an unverified Phase I; no public confirmation found; treat as speculative pending Kemah planning dept / CoStar source check</t>
+        </is>
+      </c>
+      <c r="H13" s="32" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="39" t="inlineStr">
+        <is>
+          <t>Property / Site</t>
+        </is>
+      </c>
+      <c r="C16" s="39" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="inlineStr">
+        <is>
+          <t>Est. Delivery</t>
+        </is>
+      </c>
+      <c r="E16" s="39" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F16" s="39" t="inlineStr">
+        <is>
+          <t>Leasing Pace</t>
+        </is>
+      </c>
+      <c r="G16" s="39" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="H16" s="39" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Westland Ranch MPC potential MF tract</t>
+        </is>
+      </c>
+      <c r="C17" s="62" t="n"/>
+      <c r="D17" s="62" t="n"/>
+      <c r="E17" s="32" t="inlineStr">
+        <is>
+          <t>planned/speculative</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="n"/>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>Meritage Homes MPC, W League City near SH-99/FM-517 (~5-6 mi, radius edge); ~1,200+ SF lots; no confirmed apartment phase but large MPCs often carry MF tracts; MF entitlement UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="H17" s="32" t="inlineStr">
+        <is>
+          <t>https://www.meritagehomes.com/state/tx/houston/westland-ranch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>FM-518 / Main St corridor mixed-use capacity</t>
+        </is>
+      </c>
+      <c r="C18" s="62" t="n"/>
+      <c r="D18" s="62" t="n"/>
+      <c r="E18" s="32" t="inlineStr">
+        <is>
+          <t>zoning/entitlement capacity</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="n"/>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>League City comp plan &amp; recent rezonings along FM-518 favor mixed-use w/ residential (The League sits here); latent MF capacity exists but no specific unnamed funded project confirmed</t>
+        </is>
+      </c>
+      <c r="H18" s="32" t="inlineStr">
+        <is>
+          <t>https://www.leaguecitytx.gov/151/Planning</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>Webster / SH-3 &amp; Bay Area Blvd MF node</t>
+        </is>
+      </c>
+      <c r="C19" s="62" t="n"/>
+      <c r="D19" s="62" t="n"/>
+      <c r="E19" s="32" t="inlineStr">
+        <is>
+          <t>redevelopment node</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="n"/>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>Webster (Baybrook/I-45 hub, ~4-5 mi N) actively courts MF; OHT/Crow 336u JV sits here; likely additional latent MF capacity but no specific unnamed verified project found</t>
+        </is>
+      </c>
+      <c r="H19" s="32" t="inlineStr">
+        <is>
+          <t>https://www.cityofwebster.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Friendswood multifamily</t>
+        </is>
+      </c>
+      <c r="C20" s="62" t="n"/>
+      <c r="D20" s="62" t="n"/>
+      <c r="E20" s="32" t="inlineStr">
+        <is>
+          <t>none confirmed</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>Friendswood largely SF-oriented, historically resistant to high-density MF; some mixed-use discussion at FM-518/FM-528 but nothing concrete; no specific latent apartment project found</t>
+        </is>
+      </c>
+      <c r="H20" s="32" t="inlineStr">
+        <is>
+          <t>not found</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B15:H15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Compute Proximity column from geocoded subject->comp distance
Factor geocoding into a shared scripts/geo.py (Locator, Nominatim with
ZIP-centroid fallback, haversine) used by both the chart and the map.
The Competitive Analysis tab now fills Proximity (mi) automatically
instead of leaving it blank; add --no-geocode for offline-only runs.
Regenerate the three example workbooks and the Aura map.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;;&quot;—&quot;"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot; mi&quot;;;&quot;—&quot;"/>
+    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -191,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -224,6 +225,9 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -243,6 +247,9 @@
     <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -260,6 +267,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -313,10 +323,10 @@
     <xf numFmtId="164" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -833,17 +843,19 @@
         </is>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.92</v>
+        <v>0.929</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1861</v>
+        <v>1439</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
           <t>LIV Development</t>
         </is>
       </c>
-      <c r="I6" s="7" t="n"/>
+      <c r="I6" s="12" t="n">
+        <v>3</v>
+      </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
@@ -873,17 +885,19 @@
         </is>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.948454</v>
+        <v>0.952</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>1897</v>
+        <v>1927</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
           <t>DRA Advisors</t>
         </is>
       </c>
-      <c r="I7" s="7" t="n"/>
+      <c r="I7" s="12" t="n">
+        <v>7.2</v>
+      </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
@@ -909,17 +923,19 @@
         </is>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.879365</v>
+        <v>0.911</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>1836</v>
+        <v>1821</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
           <t>OHT Partners</t>
         </is>
       </c>
-      <c r="I8" s="7" t="n"/>
+      <c r="I8" s="12" t="n">
+        <v>4.5</v>
+      </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
@@ -949,17 +965,19 @@
         </is>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.902778</v>
+        <v>0.95</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>1765</v>
+        <v>1793</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
           <t>Allen Harrison Company</t>
         </is>
       </c>
-      <c r="I9" s="7" t="n"/>
+      <c r="I9" s="12" t="n">
+        <v>2.8</v>
+      </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
           <t>Garden</t>
@@ -989,17 +1007,19 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.926316</v>
+        <v>0.953</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>1795</v>
+        <v>1709</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
           <t>Alliance Residential Company</t>
         </is>
       </c>
-      <c r="I10" s="7" t="n"/>
+      <c r="I10" s="12" t="n">
+        <v>4.4</v>
+      </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
@@ -1012,425 +1032,445 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="12" t="n"/>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>UNDER CONSTRUCTION (3 properties, 885 units)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Dakota at Kemah</t>
         </is>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="17" t="n">
         <v>229</v>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
       </c>
-      <c r="F13" s="17" t="n"/>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H13" s="15" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>Dakota Enterprises</t>
         </is>
       </c>
-      <c r="I13" s="14" t="n"/>
-      <c r="J13" s="14" t="inlineStr">
+      <c r="I13" s="20" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
         <is>
           <t>Garden</t>
         </is>
       </c>
-      <c r="K13" s="15" t="inlineStr">
+      <c r="K13" s="16" t="inlineStr">
         <is>
           <t>Diligence: under construction</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="n">
+      <c r="B14" s="15" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>Lenox Clear Creek</t>
         </is>
       </c>
-      <c r="D14" s="16" t="n">
+      <c r="D14" s="17" t="n">
         <v>336</v>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Q3 2027</t>
         </is>
       </c>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H14" s="15" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>OHT Partners</t>
         </is>
       </c>
-      <c r="I14" s="14" t="n"/>
-      <c r="J14" s="14" t="inlineStr">
+      <c r="I14" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" s="15" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K14" s="15" t="inlineStr">
+      <c r="K14" s="16" t="inlineStr">
         <is>
           <t>Diligence: under construction</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>The Edge at Seabrook Town Centre</t>
         </is>
       </c>
-      <c r="D15" s="16" t="n">
+      <c r="D15" s="17" t="n">
         <v>320</v>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
       </c>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="19" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H15" s="15" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>HS Development Group</t>
         </is>
       </c>
-      <c r="I15" s="14" t="n"/>
-      <c r="J15" s="14" t="inlineStr">
+      <c r="I15" s="20" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J15" s="15" t="inlineStr">
         <is>
           <t>Townhome</t>
         </is>
       </c>
-      <c r="K15" s="15" t="inlineStr">
+      <c r="K15" s="16" t="inlineStr">
         <is>
           <t>Diligence: under construction</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>PROPOSED (7 properties, 1,963 units)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="21" t="n">
+      <c r="B18" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="C18" s="22" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>The League I</t>
         </is>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="25" t="n">
         <v>304</v>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t>Q3 2026</t>
         </is>
       </c>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="25" t="inlineStr">
+      <c r="F18" s="26" t="n"/>
+      <c r="G18" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H18" s="22" t="inlineStr">
+      <c r="H18" s="24" t="inlineStr">
         <is>
           <t>MOS R.E LLC</t>
         </is>
       </c>
-      <c r="I18" s="21" t="n"/>
-      <c r="J18" s="21" t="inlineStr">
+      <c r="I18" s="28" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K18" s="22" t="inlineStr">
+      <c r="K18" s="24" t="inlineStr">
         <is>
           <t>Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="21" t="n">
+      <c r="B19" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="C19" s="22" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Riverview at Clear Creek</t>
         </is>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="25" t="n">
         <v>298</v>
       </c>
-      <c r="E19" s="21" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
       </c>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="25" t="inlineStr">
+      <c r="F19" s="26" t="n"/>
+      <c r="G19" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H19" s="22" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>Atticus Real Estate</t>
         </is>
       </c>
-      <c r="I19" s="21" t="n"/>
-      <c r="J19" s="21" t="inlineStr">
+      <c r="I19" s="28" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="J19" s="23" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K19" s="22" t="inlineStr">
+      <c r="K19" s="24" t="inlineStr">
         <is>
           <t>Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="21" t="n">
+      <c r="B20" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="C20" s="22" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>Seabrook Plaza</t>
         </is>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="25" t="n">
         <v>260</v>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="E20" s="23" t="inlineStr">
         <is>
           <t>Q3 2028</t>
         </is>
       </c>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="25" t="inlineStr">
+      <c r="F20" s="26" t="n"/>
+      <c r="G20" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H20" s="22" t="inlineStr">
+      <c r="H20" s="24" t="inlineStr">
         <is>
           <t>HM Equity Management</t>
         </is>
       </c>
-      <c r="I20" s="21" t="n"/>
-      <c r="J20" s="21" t="inlineStr">
+      <c r="I20" s="28" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J20" s="23" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K20" s="22" t="inlineStr">
+      <c r="K20" s="24" t="inlineStr">
         <is>
           <t>Units: CoStar 260 vs RealPage 76; Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="23" t="n">
         <v>12</v>
       </c>
-      <c r="C21" s="22" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>The League Future Phases</t>
         </is>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="25" t="n">
         <v>400</v>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="25" t="inlineStr">
+      <c r="F21" s="26" t="n"/>
+      <c r="G21" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H21" s="22" t="inlineStr">
+      <c r="H21" s="24" t="inlineStr">
         <is>
           <t>Privately Owned</t>
         </is>
       </c>
-      <c r="I21" s="21" t="n"/>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="I21" s="28" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J21" s="23" t="inlineStr">
         <is>
           <t>Mid-Rise</t>
         </is>
       </c>
-      <c r="K21" s="22" t="inlineStr">
+      <c r="K21" s="24" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="21" t="n">
+      <c r="B22" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>Residences at Highland Center</t>
         </is>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="25" t="n">
         <v>275</v>
       </c>
-      <c r="E22" s="21" t="inlineStr">
+      <c r="E22" s="23" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="25" t="inlineStr">
+      <c r="F22" s="26" t="n"/>
+      <c r="G22" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H22" s="22" t="inlineStr">
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>Highland Resources Inc</t>
         </is>
       </c>
-      <c r="I22" s="21" t="n"/>
-      <c r="J22" s="21" t="inlineStr">
+      <c r="I22" s="28" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J22" s="23" t="inlineStr">
         <is>
           <t>High-Rise</t>
         </is>
       </c>
-      <c r="K22" s="22" t="inlineStr">
+      <c r="K22" s="24" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="21" t="n">
+      <c r="B23" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="C23" s="22" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>Avalon at Kemah II</t>
         </is>
       </c>
-      <c r="D23" s="23" t="n">
+      <c r="D23" s="25" t="n">
         <v>228</v>
       </c>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="E23" s="23" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="25" t="inlineStr">
+      <c r="F23" s="26" t="n"/>
+      <c r="G23" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H23" s="22" t="inlineStr">
+      <c r="H23" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I23" s="21" t="n"/>
-      <c r="J23" s="21" t="inlineStr">
+      <c r="I23" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="23" t="inlineStr">
         <is>
           <t>Garden</t>
         </is>
       </c>
-      <c r="K23" s="22" t="inlineStr">
+      <c r="K23" s="24" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="21" t="n">
+      <c r="B24" s="23" t="n">
         <v>15</v>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>Avalon at Kemah I</t>
         </is>
       </c>
-      <c r="D24" s="23" t="n">
+      <c r="D24" s="25" t="n">
         <v>198</v>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F24" s="24" t="n"/>
-      <c r="G24" s="25" t="inlineStr">
+      <c r="F24" s="26" t="n"/>
+      <c r="G24" s="27" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H24" s="22" t="inlineStr">
+      <c r="H24" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I24" s="21" t="n"/>
-      <c r="J24" s="21" t="inlineStr">
+      <c r="I24" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>Garden</t>
         </is>
       </c>
-      <c r="K24" s="22" t="inlineStr">
+      <c r="K24" s="24" t="inlineStr">
         <is>
           <t>RealPage pipeline (not yet in CoStar); Diligence: proposed</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="26" t="inlineStr">
-        <is>
-          <t>* 5-Mile radius. Rent ($) = market asking. Proximity (mi) to be filled manually; lease-up rent/occupancy to be verified w/ HelloData. See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>* 5-Mile radius. Rent ($) = market asking. Proximity (mi) = straight-line distance from the subject (geocoded); lease-up rent/occupancy to be verified w/ HelloData. See the 'Supply &amp; Absorption' tab for the forward supply / absorption / overall-occupancy forecast.</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1538,7 @@
       </c>
     </row>
     <row r="3" ht="14.4" customHeight="1">
-      <c r="R3" s="27" t="inlineStr">
+      <c r="R3" s="30" t="inlineStr">
         <is>
           <t>UNDER CONSTRUCTION (linked from Competitive Analysis)</t>
         </is>
@@ -1509,52 +1549,52 @@
       </c>
     </row>
     <row r="4" ht="14.4" customHeight="1">
-      <c r="B4" s="28" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>As-of Quarter</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="32" t="inlineStr">
         <is>
           <t>Q2 2026</t>
         </is>
       </c>
-      <c r="R4" s="30" t="inlineStr">
+      <c r="R4" s="33" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="S4" s="30" t="inlineStr">
+      <c r="S4" s="33" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="T4" s="30" t="inlineStr">
+      <c r="T4" s="33" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
     </row>
     <row r="5" ht="14.4" customHeight="1">
-      <c r="B5" s="28" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>Close Quarter (Y1 start)</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="34" t="inlineStr">
         <is>
           <t>Q4 2026</t>
         </is>
       </c>
-      <c r="R5" s="32">
+      <c r="R5" s="35">
         <f>'Competitive Analysis'!C14</f>
         <v/>
       </c>
-      <c r="S5" s="33">
+      <c r="S5" s="36">
         <f>'Competitive Analysis'!D14</f>
         <v/>
       </c>
-      <c r="T5" s="34">
+      <c r="T5" s="37">
         <f>'Competitive Analysis'!E14</f>
         <v/>
       </c>
@@ -1568,23 +1608,23 @@
       </c>
     </row>
     <row r="6" ht="14.4" customHeight="1">
-      <c r="B6" s="28" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>Stabilization Target</t>
         </is>
       </c>
-      <c r="C6" s="35" t="n">
+      <c r="C6" s="38" t="n">
         <v>0.95</v>
       </c>
-      <c r="R6" s="32">
+      <c r="R6" s="35">
         <f>'Competitive Analysis'!C15</f>
         <v/>
       </c>
-      <c r="S6" s="33">
+      <c r="S6" s="36">
         <f>'Competitive Analysis'!D15</f>
         <v/>
       </c>
-      <c r="T6" s="34">
+      <c r="T6" s="37">
         <f>'Competitive Analysis'!E15</f>
         <v/>
       </c>
@@ -1598,25 +1638,25 @@
       </c>
     </row>
     <row r="7" ht="14.4" customHeight="1">
-      <c r="B7" s="28" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>Demand Scenario</t>
         </is>
       </c>
-      <c r="C7" s="31" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="R7" s="32">
+      <c r="R7" s="35">
         <f>'Competitive Analysis'!C13</f>
         <v/>
       </c>
-      <c r="S7" s="33">
+      <c r="S7" s="36">
         <f>'Competitive Analysis'!D13</f>
         <v/>
       </c>
-      <c r="T7" s="34">
+      <c r="T7" s="37">
         <f>'Competitive Analysis'!E13</f>
         <v/>
       </c>
@@ -1630,80 +1670,80 @@
       </c>
     </row>
     <row r="8" ht="14.4" customHeight="1">
-      <c r="B8" s="28" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>Bear Annual Absorption</t>
         </is>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="39" t="n">
         <v>150</v>
       </c>
     </row>
     <row r="9" ht="14.4" customHeight="1">
-      <c r="B9" s="28" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Base Annual Absorption</t>
         </is>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="39" t="n">
         <v>325</v>
       </c>
-      <c r="R9" s="27" t="inlineStr">
+      <c r="R9" s="30" t="inlineStr">
         <is>
           <t>PROPOSED PIPELINE (scenario toggle)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="14.4" customHeight="1">
-      <c r="B10" s="28" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>Bull Annual Absorption</t>
         </is>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="39" t="n">
         <v>500</v>
       </c>
-      <c r="R10" s="30" t="inlineStr">
+      <c r="R10" s="33" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="S10" s="30" t="inlineStr">
+      <c r="S10" s="33" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="T10" s="30" t="inlineStr">
+      <c r="T10" s="33" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="U10" s="30" t="inlineStr">
+      <c r="U10" s="33" t="inlineStr">
         <is>
           <t>Built In</t>
         </is>
       </c>
     </row>
     <row r="11" ht="14.4" customHeight="1">
-      <c r="B11" s="28" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>Selected Annual Demand</t>
         </is>
       </c>
-      <c r="C11" s="37">
+      <c r="C11" s="40">
         <f>IF($C$7="Bear",$C$8,IF($C$7="Bull",$C$10,$C$9))</f>
         <v/>
       </c>
-      <c r="R11" s="32" t="inlineStr">
+      <c r="R11" s="35" t="inlineStr">
         <is>
           <t>The League Future Phases</t>
         </is>
       </c>
-      <c r="S11" s="33" t="n">
+      <c r="S11" s="36" t="n">
         <v>400</v>
       </c>
-      <c r="T11" s="38" t="inlineStr"/>
-      <c r="U11" s="38" t="inlineStr">
+      <c r="T11" s="41" t="inlineStr"/>
+      <c r="U11" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1722,20 +1762,20 @@
       </c>
     </row>
     <row r="12" ht="14.4" customHeight="1">
-      <c r="R12" s="32" t="inlineStr">
+      <c r="R12" s="35" t="inlineStr">
         <is>
           <t>The League I</t>
         </is>
       </c>
-      <c r="S12" s="33" t="n">
+      <c r="S12" s="36" t="n">
         <v>304</v>
       </c>
-      <c r="T12" s="38" t="inlineStr">
+      <c r="T12" s="41" t="inlineStr">
         <is>
           <t>Q3 2026</t>
         </is>
       </c>
-      <c r="U12" s="38" t="inlineStr">
+      <c r="U12" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1754,20 +1794,20 @@
       </c>
     </row>
     <row r="13" ht="14.4" customHeight="1">
-      <c r="R13" s="32" t="inlineStr">
+      <c r="R13" s="35" t="inlineStr">
         <is>
           <t>Riverview at Clear Creek</t>
         </is>
       </c>
-      <c r="S13" s="33" t="n">
+      <c r="S13" s="36" t="n">
         <v>298</v>
       </c>
-      <c r="T13" s="38" t="inlineStr">
+      <c r="T13" s="41" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
       </c>
-      <c r="U13" s="38" t="inlineStr">
+      <c r="U13" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1786,16 +1826,16 @@
       </c>
     </row>
     <row r="14" ht="14.4" customHeight="1">
-      <c r="R14" s="32" t="inlineStr">
+      <c r="R14" s="35" t="inlineStr">
         <is>
           <t>Residences at Highland Center</t>
         </is>
       </c>
-      <c r="S14" s="33" t="n">
+      <c r="S14" s="36" t="n">
         <v>275</v>
       </c>
-      <c r="T14" s="38" t="inlineStr"/>
-      <c r="U14" s="38" t="inlineStr">
+      <c r="T14" s="41" t="inlineStr"/>
+      <c r="U14" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1814,20 +1854,20 @@
       </c>
     </row>
     <row r="15" ht="14.4" customHeight="1">
-      <c r="R15" s="32" t="inlineStr">
+      <c r="R15" s="35" t="inlineStr">
         <is>
           <t>Seabrook Plaza</t>
         </is>
       </c>
-      <c r="S15" s="33" t="n">
+      <c r="S15" s="36" t="n">
         <v>260</v>
       </c>
-      <c r="T15" s="38" t="inlineStr">
+      <c r="T15" s="41" t="inlineStr">
         <is>
           <t>Q3 2028</t>
         </is>
       </c>
-      <c r="U15" s="38" t="inlineStr">
+      <c r="U15" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1846,16 +1886,16 @@
       </c>
     </row>
     <row r="16" ht="14.4" customHeight="1">
-      <c r="R16" s="32" t="inlineStr">
+      <c r="R16" s="35" t="inlineStr">
         <is>
           <t>Avalon at Kemah II</t>
         </is>
       </c>
-      <c r="S16" s="33" t="n">
+      <c r="S16" s="36" t="n">
         <v>228</v>
       </c>
-      <c r="T16" s="38" t="inlineStr"/>
-      <c r="U16" s="38" t="inlineStr">
+      <c r="T16" s="41" t="inlineStr"/>
+      <c r="U16" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1874,7 +1914,7 @@
       </c>
     </row>
     <row r="17" ht="14.4" customHeight="1">
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>5-MILE MARKET</t>
         </is>
@@ -1914,46 +1954,46 @@
           <t>Y0</t>
         </is>
       </c>
-      <c r="J17" s="39" t="inlineStr">
+      <c r="J17" s="42" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K17" s="39" t="inlineStr">
+      <c r="K17" s="42" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L17" s="39" t="inlineStr">
+      <c r="L17" s="42" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M17" s="39" t="inlineStr">
+      <c r="M17" s="42" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N17" s="39" t="inlineStr">
+      <c r="N17" s="42" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O17" s="39" t="inlineStr">
+      <c r="O17" s="42" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
-      <c r="R17" s="32" t="inlineStr">
+      <c r="R17" s="35" t="inlineStr">
         <is>
           <t>Avalon at Kemah I</t>
         </is>
       </c>
-      <c r="S17" s="33" t="n">
+      <c r="S17" s="36" t="n">
         <v>198</v>
       </c>
-      <c r="T17" s="38" t="inlineStr"/>
-      <c r="U17" s="38" t="inlineStr">
+      <c r="T17" s="41" t="inlineStr"/>
+      <c r="U17" s="41" t="inlineStr">
         <is>
           <t>Bear only</t>
         </is>
@@ -1972,1064 +2012,1064 @@
       </c>
     </row>
     <row r="18" ht="14.4" customHeight="1">
-      <c r="C18" s="40" t="inlineStr">
+      <c r="C18" s="43" t="inlineStr">
         <is>
           <t>Q3'19-Q2'20</t>
         </is>
       </c>
-      <c r="D18" s="40" t="inlineStr">
+      <c r="D18" s="43" t="inlineStr">
         <is>
           <t>Q3'20-Q2'21</t>
         </is>
       </c>
-      <c r="E18" s="40" t="inlineStr">
+      <c r="E18" s="43" t="inlineStr">
         <is>
           <t>Q3'21-Q2'22</t>
         </is>
       </c>
-      <c r="F18" s="40" t="inlineStr">
+      <c r="F18" s="43" t="inlineStr">
         <is>
           <t>Q3'22-Q2'23</t>
         </is>
       </c>
-      <c r="G18" s="40" t="inlineStr">
+      <c r="G18" s="43" t="inlineStr">
         <is>
           <t>Q3'23-Q2'24</t>
         </is>
       </c>
-      <c r="H18" s="40" t="inlineStr">
+      <c r="H18" s="43" t="inlineStr">
         <is>
           <t>Q3'24-Q2'25</t>
         </is>
       </c>
-      <c r="I18" s="40" t="inlineStr">
+      <c r="I18" s="43" t="inlineStr">
         <is>
           <t>Q3'25-Q2'26</t>
         </is>
       </c>
-      <c r="J18" s="40" t="inlineStr">
+      <c r="J18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 1</t>
         </is>
       </c>
-      <c r="K18" s="40" t="inlineStr">
+      <c r="K18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 2</t>
         </is>
       </c>
-      <c r="L18" s="40" t="inlineStr">
+      <c r="L18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 3</t>
         </is>
       </c>
-      <c r="M18" s="40" t="inlineStr">
+      <c r="M18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 4</t>
         </is>
       </c>
-      <c r="N18" s="40" t="inlineStr">
+      <c r="N18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 5</t>
         </is>
       </c>
-      <c r="O18" s="40" t="inlineStr">
+      <c r="O18" s="43" t="inlineStr">
         <is>
           <t>Hold Yr 6</t>
         </is>
       </c>
     </row>
     <row r="19" ht="14.4" customHeight="1">
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>NEW SUPPLY (5-mi)</t>
         </is>
       </c>
-      <c r="C19" s="41" t="n">
+      <c r="C19" s="44" t="n">
         <v>351</v>
       </c>
-      <c r="D19" s="41" t="n">
+      <c r="D19" s="44" t="n">
         <v>656</v>
       </c>
-      <c r="E19" s="41" t="n">
+      <c r="E19" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="41" t="n">
+      <c r="F19" s="44" t="n">
         <v>1221</v>
       </c>
-      <c r="G19" s="41" t="n">
+      <c r="G19" s="44" t="n">
         <v>360</v>
       </c>
-      <c r="H19" s="41" t="n">
+      <c r="H19" s="44" t="n">
         <v>380</v>
       </c>
-      <c r="I19" s="41" t="n">
+      <c r="I19" s="44" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="42">
+      <c r="J19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,1)+SUMIFS($S$11:$S$17,$W$11:$W$17,1,$X$11:$X$17,1)</f>
         <v/>
       </c>
-      <c r="K19" s="42">
+      <c r="K19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,2)+SUMIFS($S$11:$S$17,$W$11:$W$17,2,$X$11:$X$17,1)</f>
         <v/>
       </c>
-      <c r="L19" s="42">
+      <c r="L19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,3)+SUMIFS($S$11:$S$17,$W$11:$W$17,3,$X$11:$X$17,1)</f>
         <v/>
       </c>
-      <c r="M19" s="42">
+      <c r="M19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,4)+SUMIFS($S$11:$S$17,$W$11:$W$17,4,$X$11:$X$17,1)</f>
         <v/>
       </c>
-      <c r="N19" s="42">
+      <c r="N19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,5)+SUMIFS($S$11:$S$17,$W$11:$W$17,5,$X$11:$X$17,1)</f>
         <v/>
       </c>
-      <c r="O19" s="42">
+      <c r="O19" s="45">
         <f>SUMIFS($S$5:$S$7,$W$5:$W$7,6)+SUMIFS($S$11:$S$17,$W$11:$W$17,6,$X$11:$X$17,1)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="14.4" customHeight="1">
-      <c r="B20" s="28" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>ABSORPTION (5-mi)</t>
         </is>
       </c>
-      <c r="C20" s="41" t="n">
+      <c r="C20" s="44" t="n">
         <v>262</v>
       </c>
-      <c r="D20" s="41" t="n">
+      <c r="D20" s="44" t="n">
         <v>800</v>
       </c>
-      <c r="E20" s="41" t="n">
+      <c r="E20" s="44" t="n">
         <v>-336</v>
       </c>
-      <c r="F20" s="41" t="n">
+      <c r="F20" s="44" t="n">
         <v>458</v>
       </c>
-      <c r="G20" s="41" t="n">
+      <c r="G20" s="44" t="n">
         <v>575</v>
       </c>
-      <c r="H20" s="41" t="n">
+      <c r="H20" s="44" t="n">
         <v>501</v>
       </c>
-      <c r="I20" s="41" t="n">
+      <c r="I20" s="44" t="n">
         <v>-74</v>
       </c>
-      <c r="J20" s="42">
+      <c r="J20" s="45">
         <f>J31-I31</f>
         <v/>
       </c>
-      <c r="K20" s="42">
+      <c r="K20" s="45">
         <f>K31-J31</f>
         <v/>
       </c>
-      <c r="L20" s="42">
+      <c r="L20" s="45">
         <f>L31-K31</f>
         <v/>
       </c>
-      <c r="M20" s="42">
+      <c r="M20" s="45">
         <f>M31-L31</f>
         <v/>
       </c>
-      <c r="N20" s="42">
+      <c r="N20" s="45">
         <f>N31-M31</f>
         <v/>
       </c>
-      <c r="O20" s="42">
+      <c r="O20" s="45">
         <f>O31-N31</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="14.4" customHeight="1">
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>OCCUPANCY (5-mi)</t>
         </is>
       </c>
-      <c r="C21" s="43" t="n">
+      <c r="C21" s="46" t="n">
         <v>0.925</v>
       </c>
-      <c r="D21" s="43" t="n">
+      <c r="D21" s="46" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="E21" s="43" t="n">
+      <c r="E21" s="46" t="n">
         <v>0.919</v>
       </c>
-      <c r="F21" s="43" t="n">
+      <c r="F21" s="46" t="n">
         <v>0.892</v>
       </c>
-      <c r="G21" s="43" t="n">
+      <c r="G21" s="46" t="n">
         <v>0.902</v>
       </c>
-      <c r="H21" s="43" t="n">
+      <c r="H21" s="46" t="n">
         <v>0.908</v>
       </c>
-      <c r="I21" s="43" t="n">
+      <c r="I21" s="46" t="n">
         <v>0.905</v>
       </c>
-      <c r="J21" s="44">
+      <c r="J21" s="47">
         <f>IFERROR(J31/J30,0)</f>
         <v/>
       </c>
-      <c r="K21" s="44">
+      <c r="K21" s="47">
         <f>IFERROR(K31/K30,0)</f>
         <v/>
       </c>
-      <c r="L21" s="44">
+      <c r="L21" s="47">
         <f>IFERROR(L31/L30,0)</f>
         <v/>
       </c>
-      <c r="M21" s="44">
+      <c r="M21" s="47">
         <f>IFERROR(M31/M30,0)</f>
         <v/>
       </c>
-      <c r="N21" s="44">
+      <c r="N21" s="47">
         <f>IFERROR(N31/N30,0)</f>
         <v/>
       </c>
-      <c r="O21" s="44">
+      <c r="O21" s="47">
         <f>IFERROR(O31/O30,0)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="14.4" customHeight="1">
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="31" t="inlineStr">
         <is>
           <t>SUBJECT (Aura Beacon Island)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="14.4" customHeight="1">
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Market Rent  (RealPage→HD)</t>
         </is>
       </c>
-      <c r="C23" s="45" t="n"/>
-      <c r="D23" s="45" t="n"/>
-      <c r="E23" s="45" t="n"/>
-      <c r="F23" s="45" t="n">
+      <c r="C23" s="48" t="n"/>
+      <c r="D23" s="48" t="n"/>
+      <c r="E23" s="48" t="n"/>
+      <c r="F23" s="48" t="n">
         <v>1795</v>
       </c>
-      <c r="G23" s="45" t="n">
+      <c r="G23" s="48" t="n">
         <v>1854</v>
       </c>
-      <c r="H23" s="45" t="n">
+      <c r="H23" s="48" t="n">
         <v>1793</v>
       </c>
-      <c r="I23" s="45" t="n">
+      <c r="I23" s="48" t="n">
         <v>1782</v>
       </c>
-      <c r="J23" s="46" t="n"/>
-      <c r="K23" s="46" t="n"/>
-      <c r="L23" s="46" t="n"/>
-      <c r="M23" s="46" t="n"/>
-      <c r="N23" s="46" t="n"/>
-      <c r="O23" s="46" t="n"/>
+      <c r="J23" s="49" t="n"/>
+      <c r="K23" s="49" t="n"/>
+      <c r="L23" s="49" t="n"/>
+      <c r="M23" s="49" t="n"/>
+      <c r="N23" s="49" t="n"/>
+      <c r="O23" s="49" t="n"/>
     </row>
     <row r="24" ht="14.4" customHeight="1">
-      <c r="B24" s="47" t="inlineStr">
+      <c r="B24" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">    Market Rent YoY %</t>
         </is>
       </c>
-      <c r="C24" s="48" t="n"/>
-      <c r="D24" s="48">
+      <c r="C24" s="51" t="n"/>
+      <c r="D24" s="51">
         <f>IFERROR(D23/C23-1,"")</f>
         <v/>
       </c>
-      <c r="E24" s="48">
+      <c r="E24" s="51">
         <f>IFERROR(E23/D23-1,"")</f>
         <v/>
       </c>
-      <c r="F24" s="48">
+      <c r="F24" s="51">
         <f>IFERROR(F23/E23-1,"")</f>
         <v/>
       </c>
-      <c r="G24" s="48">
+      <c r="G24" s="51">
         <f>IFERROR(G23/F23-1,"")</f>
         <v/>
       </c>
-      <c r="H24" s="48">
+      <c r="H24" s="51">
         <f>IFERROR(H23/G23-1,"")</f>
         <v/>
       </c>
-      <c r="I24" s="48">
+      <c r="I24" s="51">
         <f>IFERROR(I23/H23-1,"")</f>
         <v/>
       </c>
-      <c r="J24" s="49" t="n"/>
-      <c r="K24" s="49" t="n"/>
-      <c r="L24" s="49" t="n"/>
-      <c r="M24" s="49" t="n"/>
-      <c r="N24" s="49" t="n"/>
-      <c r="O24" s="49" t="n"/>
+      <c r="J24" s="52" t="n"/>
+      <c r="K24" s="52" t="n"/>
+      <c r="L24" s="52" t="n"/>
+      <c r="M24" s="52" t="n"/>
+      <c r="N24" s="52" t="n"/>
+      <c r="O24" s="52" t="n"/>
     </row>
     <row r="25" ht="14.4" customHeight="1">
-      <c r="B25" s="28" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Effective Rent</t>
         </is>
       </c>
-      <c r="C25" s="45" t="n"/>
-      <c r="D25" s="45" t="n"/>
-      <c r="E25" s="45" t="n"/>
-      <c r="F25" s="45" t="n">
+      <c r="C25" s="48" t="n"/>
+      <c r="D25" s="48" t="n"/>
+      <c r="E25" s="48" t="n"/>
+      <c r="F25" s="48" t="n">
         <v>1657</v>
       </c>
-      <c r="G25" s="45" t="n">
+      <c r="G25" s="48" t="n">
         <v>1728</v>
       </c>
-      <c r="H25" s="45" t="n">
+      <c r="H25" s="48" t="n">
         <v>1697</v>
       </c>
-      <c r="I25" s="45" t="n">
+      <c r="I25" s="48" t="n">
         <v>1543</v>
       </c>
-      <c r="J25" s="46" t="n"/>
-      <c r="K25" s="46" t="n"/>
-      <c r="L25" s="46" t="n"/>
-      <c r="M25" s="46" t="n"/>
-      <c r="N25" s="46" t="n"/>
-      <c r="O25" s="46" t="n"/>
+      <c r="J25" s="49" t="n"/>
+      <c r="K25" s="49" t="n"/>
+      <c r="L25" s="49" t="n"/>
+      <c r="M25" s="49" t="n"/>
+      <c r="N25" s="49" t="n"/>
+      <c r="O25" s="49" t="n"/>
     </row>
     <row r="26" ht="14.4" customHeight="1">
-      <c r="B26" s="47" t="inlineStr">
+      <c r="B26" s="50" t="inlineStr">
         <is>
           <t xml:space="preserve">    Effective Rent YoY %</t>
         </is>
       </c>
-      <c r="C26" s="48" t="n"/>
-      <c r="D26" s="48">
+      <c r="C26" s="51" t="n"/>
+      <c r="D26" s="51">
         <f>IFERROR(D25/C25-1,"")</f>
         <v/>
       </c>
-      <c r="E26" s="48">
+      <c r="E26" s="51">
         <f>IFERROR(E25/D25-1,"")</f>
         <v/>
       </c>
-      <c r="F26" s="48">
+      <c r="F26" s="51">
         <f>IFERROR(F25/E25-1,"")</f>
         <v/>
       </c>
-      <c r="G26" s="48">
+      <c r="G26" s="51">
         <f>IFERROR(G25/F25-1,"")</f>
         <v/>
       </c>
-      <c r="H26" s="48">
+      <c r="H26" s="51">
         <f>IFERROR(H25/G25-1,"")</f>
         <v/>
       </c>
-      <c r="I26" s="48">
+      <c r="I26" s="51">
         <f>IFERROR(I25/H25-1,"")</f>
         <v/>
       </c>
-      <c r="J26" s="49" t="n"/>
-      <c r="K26" s="49" t="n"/>
-      <c r="L26" s="49" t="n"/>
-      <c r="M26" s="49" t="n"/>
-      <c r="N26" s="49" t="n"/>
-      <c r="O26" s="49" t="n"/>
+      <c r="J26" s="52" t="n"/>
+      <c r="K26" s="52" t="n"/>
+      <c r="L26" s="52" t="n"/>
+      <c r="M26" s="52" t="n"/>
+      <c r="N26" s="52" t="n"/>
+      <c r="O26" s="52" t="n"/>
     </row>
     <row r="27" ht="14.4" customHeight="1">
-      <c r="B27" s="28" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Occupancy (financials / CoStar)</t>
         </is>
       </c>
-      <c r="C27" s="50" t="n"/>
-      <c r="D27" s="50" t="n"/>
-      <c r="E27" s="50" t="n"/>
-      <c r="F27" s="50" t="n">
+      <c r="C27" s="53" t="n"/>
+      <c r="D27" s="53" t="n"/>
+      <c r="E27" s="53" t="n"/>
+      <c r="F27" s="53" t="n">
         <v>0.3413793103448277</v>
       </c>
-      <c r="G27" s="50" t="n">
+      <c r="G27" s="53" t="n">
         <v>0.8775862068965519</v>
       </c>
-      <c r="H27" s="50" t="n">
+      <c r="H27" s="53" t="n">
         <v>0.9324033975977525</v>
       </c>
-      <c r="I27" s="50" t="n">
+      <c r="I27" s="53" t="n">
         <v>0.9194867500515453</v>
       </c>
-      <c r="J27" s="51" t="n"/>
-      <c r="K27" s="51" t="n"/>
-      <c r="L27" s="51" t="n"/>
-      <c r="M27" s="51" t="n"/>
-      <c r="N27" s="51" t="n"/>
-      <c r="O27" s="51" t="n"/>
+      <c r="J27" s="54" t="n"/>
+      <c r="K27" s="54" t="n"/>
+      <c r="L27" s="54" t="n"/>
+      <c r="M27" s="54" t="n"/>
+      <c r="N27" s="54" t="n"/>
+      <c r="O27" s="54" t="n"/>
     </row>
     <row r="28" ht="14.4" customHeight="1">
-      <c r="B28" s="28" t="inlineStr">
+      <c r="B28" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Concession %</t>
         </is>
       </c>
-      <c r="C28" s="50" t="n"/>
-      <c r="D28" s="50" t="n"/>
-      <c r="E28" s="50" t="n"/>
-      <c r="F28" s="50">
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="53">
         <f>IFERROR((F23-F25)/F23,"")</f>
         <v/>
       </c>
-      <c r="G28" s="50">
+      <c r="G28" s="53">
         <f>IFERROR((G23-G25)/G23,"")</f>
         <v/>
       </c>
-      <c r="H28" s="50">
+      <c r="H28" s="53">
         <f>IFERROR((H23-H25)/H23,"")</f>
         <v/>
       </c>
-      <c r="I28" s="50">
+      <c r="I28" s="53">
         <f>IFERROR((I23-I25)/I23,"")</f>
         <v/>
       </c>
-      <c r="J28" s="51" t="n"/>
-      <c r="K28" s="51" t="n"/>
-      <c r="L28" s="51" t="n"/>
-      <c r="M28" s="51" t="n"/>
-      <c r="N28" s="51" t="n"/>
-      <c r="O28" s="51" t="n"/>
+      <c r="J28" s="54" t="n"/>
+      <c r="K28" s="54" t="n"/>
+      <c r="L28" s="54" t="n"/>
+      <c r="M28" s="54" t="n"/>
+      <c r="N28" s="54" t="n"/>
+      <c r="O28" s="54" t="n"/>
     </row>
     <row r="29" ht="14.4" customHeight="1"/>
     <row r="30" hidden="1" ht="14.4" customHeight="1">
-      <c r="B30" s="26" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  inventory</t>
         </is>
       </c>
-      <c r="C30" s="52" t="n">
+      <c r="C30" s="55" t="n">
         <v>23134</v>
       </c>
-      <c r="D30" s="52" t="n">
+      <c r="D30" s="55" t="n">
         <v>23790</v>
       </c>
-      <c r="E30" s="52" t="n">
+      <c r="E30" s="55" t="n">
         <v>23790</v>
       </c>
-      <c r="F30" s="52" t="n">
+      <c r="F30" s="55" t="n">
         <v>25011</v>
       </c>
-      <c r="G30" s="52" t="n">
+      <c r="G30" s="55" t="n">
         <v>25371</v>
       </c>
-      <c r="H30" s="52" t="n">
+      <c r="H30" s="55" t="n">
         <v>25751</v>
       </c>
-      <c r="I30" s="52" t="n">
+      <c r="I30" s="55" t="n">
         <v>25751</v>
       </c>
-      <c r="J30" s="52">
+      <c r="J30" s="55">
         <f>I30+J19</f>
         <v/>
       </c>
-      <c r="K30" s="52">
+      <c r="K30" s="55">
         <f>J30+K19</f>
         <v/>
       </c>
-      <c r="L30" s="52">
+      <c r="L30" s="55">
         <f>K30+L19</f>
         <v/>
       </c>
-      <c r="M30" s="52">
+      <c r="M30" s="55">
         <f>L30+M19</f>
         <v/>
       </c>
-      <c r="N30" s="52">
+      <c r="N30" s="55">
         <f>M30+N19</f>
         <v/>
       </c>
-      <c r="O30" s="52">
+      <c r="O30" s="55">
         <f>N30+O19</f>
         <v/>
       </c>
     </row>
     <row r="31" hidden="1" ht="14.4" customHeight="1">
-      <c r="B31" s="26" t="inlineStr">
+      <c r="B31" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  occupied</t>
         </is>
       </c>
-      <c r="C31" s="52" t="n">
+      <c r="C31" s="55" t="n">
         <v>21391</v>
       </c>
-      <c r="D31" s="52" t="n">
+      <c r="D31" s="55" t="n">
         <v>22191</v>
       </c>
-      <c r="E31" s="52" t="n">
+      <c r="E31" s="55" t="n">
         <v>21855</v>
       </c>
-      <c r="F31" s="52" t="n">
+      <c r="F31" s="55" t="n">
         <v>22313</v>
       </c>
-      <c r="G31" s="52" t="n">
+      <c r="G31" s="55" t="n">
         <v>22888</v>
       </c>
-      <c r="H31" s="52" t="n">
+      <c r="H31" s="55" t="n">
         <v>23388</v>
       </c>
-      <c r="I31" s="52" t="n">
+      <c r="I31" s="55" t="n">
         <v>23314</v>
       </c>
-      <c r="J31" s="52">
+      <c r="J31" s="55">
         <f>MIN($C$6*J30,I31+$C$11)</f>
         <v/>
       </c>
-      <c r="K31" s="52">
+      <c r="K31" s="55">
         <f>MIN($C$6*K30,J31+$C$11)</f>
         <v/>
       </c>
-      <c r="L31" s="52">
+      <c r="L31" s="55">
         <f>MIN($C$6*L30,K31+$C$11)</f>
         <v/>
       </c>
-      <c r="M31" s="52">
+      <c r="M31" s="55">
         <f>MIN($C$6*M30,L31+$C$11)</f>
         <v/>
       </c>
-      <c r="N31" s="52">
+      <c r="N31" s="55">
         <f>MIN($C$6*N30,M31+$C$11)</f>
         <v/>
       </c>
-      <c r="O31" s="52">
+      <c r="O31" s="55">
         <f>MIN($C$6*O30,N31+$C$11)</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="14.4" customHeight="1"/>
     <row r="33" ht="14.4" customHeight="1">
-      <c r="B33" s="28" t="inlineStr">
+      <c r="B33" s="31" t="inlineStr">
         <is>
           <t>IMPLIED 5-MI OCCUPANCY BY DEMAND SCENARIO</t>
         </is>
       </c>
-      <c r="J33" s="53" t="inlineStr">
+      <c r="J33" s="56" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K33" s="53" t="inlineStr">
+      <c r="K33" s="56" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L33" s="53" t="inlineStr">
+      <c r="L33" s="56" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M33" s="53" t="inlineStr">
+      <c r="M33" s="56" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N33" s="53" t="inlineStr">
+      <c r="N33" s="56" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O33" s="53" t="inlineStr">
+      <c r="O33" s="56" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
     <row r="34" ht="14.4" customHeight="1">
-      <c r="B34" s="28" t="inlineStr">
+      <c r="B34" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J34" s="54">
+      <c r="J34" s="57">
         <f>MIN($C$6,($I$31+$C$8*1)/J30)</f>
         <v/>
       </c>
-      <c r="K34" s="54">
+      <c r="K34" s="57">
         <f>MIN($C$6,($I$31+$C$8*2)/K30)</f>
         <v/>
       </c>
-      <c r="L34" s="54">
+      <c r="L34" s="57">
         <f>MIN($C$6,($I$31+$C$8*3)/L30)</f>
         <v/>
       </c>
-      <c r="M34" s="54">
+      <c r="M34" s="57">
         <f>MIN($C$6,($I$31+$C$8*4)/M30)</f>
         <v/>
       </c>
-      <c r="N34" s="54">
+      <c r="N34" s="57">
         <f>MIN($C$6,($I$31+$C$8*5)/N30)</f>
         <v/>
       </c>
-      <c r="O34" s="54">
+      <c r="O34" s="57">
         <f>MIN($C$6,($I$31+$C$8*6)/O30)</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="14.4" customHeight="1">
-      <c r="B35" s="28" t="inlineStr">
+      <c r="B35" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J35" s="54">
+      <c r="J35" s="57">
         <f>MIN($C$6,($I$31+$C$9*1)/J30)</f>
         <v/>
       </c>
-      <c r="K35" s="54">
+      <c r="K35" s="57">
         <f>MIN($C$6,($I$31+$C$9*2)/K30)</f>
         <v/>
       </c>
-      <c r="L35" s="54">
+      <c r="L35" s="57">
         <f>MIN($C$6,($I$31+$C$9*3)/L30)</f>
         <v/>
       </c>
-      <c r="M35" s="54">
+      <c r="M35" s="57">
         <f>MIN($C$6,($I$31+$C$9*4)/M30)</f>
         <v/>
       </c>
-      <c r="N35" s="54">
+      <c r="N35" s="57">
         <f>MIN($C$6,($I$31+$C$9*5)/N30)</f>
         <v/>
       </c>
-      <c r="O35" s="54">
+      <c r="O35" s="57">
         <f>MIN($C$6,($I$31+$C$9*6)/O30)</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="14.4" customHeight="1">
-      <c r="B36" s="28" t="inlineStr">
+      <c r="B36" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J36" s="54">
+      <c r="J36" s="57">
         <f>MIN($C$6,($I$31+$C$10*1)/J30)</f>
         <v/>
       </c>
-      <c r="K36" s="54">
+      <c r="K36" s="57">
         <f>MIN($C$6,($I$31+$C$10*2)/K30)</f>
         <v/>
       </c>
-      <c r="L36" s="54">
+      <c r="L36" s="57">
         <f>MIN($C$6,($I$31+$C$10*3)/L30)</f>
         <v/>
       </c>
-      <c r="M36" s="54">
+      <c r="M36" s="57">
         <f>MIN($C$6,($I$31+$C$10*4)/M30)</f>
         <v/>
       </c>
-      <c r="N36" s="54">
+      <c r="N36" s="57">
         <f>MIN($C$6,($I$31+$C$10*5)/N30)</f>
         <v/>
       </c>
-      <c r="O36" s="54">
+      <c r="O36" s="57">
         <f>MIN($C$6,($I$31+$C$10*6)/O30)</f>
         <v/>
       </c>
     </row>
     <row r="37" ht="14.4" customHeight="1"/>
     <row r="38" ht="14.4" customHeight="1">
-      <c r="B38" s="28" t="inlineStr">
+      <c r="B38" s="31" t="inlineStr">
         <is>
           <t>MARKET RENT GROWTH (editable assumptions)</t>
         </is>
       </c>
-      <c r="J38" s="55" t="inlineStr">
+      <c r="J38" s="58" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K38" s="55" t="inlineStr">
+      <c r="K38" s="58" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L38" s="55" t="inlineStr">
+      <c r="L38" s="58" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M38" s="55" t="inlineStr">
+      <c r="M38" s="58" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N38" s="55" t="inlineStr">
+      <c r="N38" s="58" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O38" s="55" t="inlineStr">
+      <c r="O38" s="58" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
     <row r="39" ht="14.4" customHeight="1">
-      <c r="B39" s="28" t="inlineStr">
+      <c r="B39" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J39" s="56" t="n">
+      <c r="J39" s="59" t="n">
         <v>-0.0025</v>
       </c>
-      <c r="K39" s="56" t="n">
+      <c r="K39" s="59" t="n">
         <v>0.0175</v>
       </c>
-      <c r="L39" s="56" t="n">
+      <c r="L39" s="59" t="n">
         <v>0.0275</v>
       </c>
-      <c r="M39" s="56" t="n">
+      <c r="M39" s="59" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N39" s="56" t="n">
+      <c r="N39" s="59" t="n">
         <v>0.0275</v>
       </c>
-      <c r="O39" s="56" t="n">
+      <c r="O39" s="59" t="n">
         <v>0.0175</v>
       </c>
     </row>
     <row r="40" ht="14.4" customHeight="1">
-      <c r="B40" s="28" t="inlineStr">
+      <c r="B40" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J40" s="56" t="n">
+      <c r="J40" s="59" t="n">
         <v>0.01</v>
       </c>
-      <c r="K40" s="56" t="n">
+      <c r="K40" s="59" t="n">
         <v>0.03</v>
       </c>
-      <c r="L40" s="56" t="n">
+      <c r="L40" s="59" t="n">
         <v>0.04</v>
       </c>
-      <c r="M40" s="56" t="n">
+      <c r="M40" s="59" t="n">
         <v>0.05</v>
       </c>
-      <c r="N40" s="56" t="n">
+      <c r="N40" s="59" t="n">
         <v>0.04</v>
       </c>
-      <c r="O40" s="56" t="n">
+      <c r="O40" s="59" t="n">
         <v>0.03</v>
       </c>
     </row>
     <row r="41" ht="14.4" customHeight="1">
-      <c r="B41" s="28" t="inlineStr">
+      <c r="B41" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J41" s="56" t="n">
+      <c r="J41" s="59" t="n">
         <v>0.02</v>
       </c>
-      <c r="K41" s="56" t="n">
+      <c r="K41" s="59" t="n">
         <v>0.04</v>
       </c>
-      <c r="L41" s="56" t="n">
+      <c r="L41" s="59" t="n">
         <v>0.05</v>
       </c>
-      <c r="M41" s="56" t="n">
+      <c r="M41" s="59" t="n">
         <v>0.06</v>
       </c>
-      <c r="N41" s="56" t="n">
+      <c r="N41" s="59" t="n">
         <v>0.05</v>
       </c>
-      <c r="O41" s="56" t="n">
+      <c r="O41" s="59" t="n">
         <v>0.04</v>
       </c>
     </row>
     <row r="42" ht="14.4" customHeight="1">
-      <c r="B42" s="28" t="inlineStr">
+      <c r="B42" s="31" t="inlineStr">
         <is>
           <t>CONCESSIONS % — forward assumption (editable)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="14.4" customHeight="1">
-      <c r="B43" s="28" t="inlineStr">
+      <c r="B43" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J43" s="56" t="n">
+      <c r="J43" s="59" t="n">
         <v>0.06</v>
       </c>
-      <c r="K43" s="56" t="n">
+      <c r="K43" s="59" t="n">
         <v>0.045</v>
       </c>
-      <c r="L43" s="56" t="n">
+      <c r="L43" s="59" t="n">
         <v>0.035</v>
       </c>
-      <c r="M43" s="56" t="n">
+      <c r="M43" s="59" t="n">
         <v>0.035</v>
       </c>
-      <c r="N43" s="56" t="n">
+      <c r="N43" s="59" t="n">
         <v>0.035</v>
       </c>
-      <c r="O43" s="56" t="n">
+      <c r="O43" s="59" t="n">
         <v>0.035</v>
       </c>
     </row>
     <row r="44" ht="14.4" customHeight="1">
-      <c r="B44" s="28" t="inlineStr">
+      <c r="B44" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J44" s="56" t="n">
+      <c r="J44" s="59" t="n">
         <v>0.03</v>
       </c>
-      <c r="K44" s="56" t="n">
+      <c r="K44" s="59" t="n">
         <v>0.015</v>
       </c>
-      <c r="L44" s="56" t="n">
+      <c r="L44" s="59" t="n">
         <v>0.005</v>
       </c>
-      <c r="M44" s="56" t="n">
+      <c r="M44" s="59" t="n">
         <v>0.005</v>
       </c>
-      <c r="N44" s="56" t="n">
+      <c r="N44" s="59" t="n">
         <v>0.005</v>
       </c>
-      <c r="O44" s="56" t="n">
+      <c r="O44" s="59" t="n">
         <v>0.005</v>
       </c>
     </row>
     <row r="45" ht="14.4" customHeight="1">
-      <c r="B45" s="28" t="inlineStr">
+      <c r="B45" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J45" s="56" t="n">
+      <c r="J45" s="59" t="n">
         <v>0.02</v>
       </c>
-      <c r="K45" s="56" t="n">
+      <c r="K45" s="59" t="n">
         <v>0.005</v>
       </c>
-      <c r="L45" s="56" t="n">
+      <c r="L45" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="M45" s="56" t="n">
+      <c r="M45" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="56" t="n">
+      <c r="N45" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="O45" s="56" t="n">
+      <c r="O45" s="59" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="46" ht="14.4" customHeight="1">
-      <c r="B46" s="28" t="inlineStr">
+      <c r="B46" s="31" t="inlineStr">
         <is>
           <t>EFFECTIVE RENT GROWTH (derived)</t>
         </is>
       </c>
     </row>
     <row r="47" ht="14.4" customHeight="1">
-      <c r="B47" s="28" t="inlineStr">
+      <c r="B47" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J47" s="54">
+      <c r="J47" s="57">
         <f>(1+J39)*(1-J43)-1</f>
         <v/>
       </c>
-      <c r="K47" s="54">
+      <c r="K47" s="57">
         <f>(1+K39)*(1-K43)/(1-J43)-1</f>
         <v/>
       </c>
-      <c r="L47" s="54">
+      <c r="L47" s="57">
         <f>(1+L39)*(1-L43)/(1-K43)-1</f>
         <v/>
       </c>
-      <c r="M47" s="54">
+      <c r="M47" s="57">
         <f>(1+M39)*(1-M43)/(1-L43)-1</f>
         <v/>
       </c>
-      <c r="N47" s="54">
+      <c r="N47" s="57">
         <f>(1+N39)*(1-N43)/(1-M43)-1</f>
         <v/>
       </c>
-      <c r="O47" s="54">
+      <c r="O47" s="57">
         <f>(1+O39)*(1-O43)/(1-N43)-1</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="14.4" customHeight="1">
-      <c r="B48" s="28" t="inlineStr">
+      <c r="B48" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J48" s="54">
+      <c r="J48" s="57">
         <f>(1+J40)*(1-J44)-1</f>
         <v/>
       </c>
-      <c r="K48" s="54">
+      <c r="K48" s="57">
         <f>(1+K40)*(1-K44)/(1-J44)-1</f>
         <v/>
       </c>
-      <c r="L48" s="54">
+      <c r="L48" s="57">
         <f>(1+L40)*(1-L44)/(1-K44)-1</f>
         <v/>
       </c>
-      <c r="M48" s="54">
+      <c r="M48" s="57">
         <f>(1+M40)*(1-M44)/(1-L44)-1</f>
         <v/>
       </c>
-      <c r="N48" s="54">
+      <c r="N48" s="57">
         <f>(1+N40)*(1-N44)/(1-M44)-1</f>
         <v/>
       </c>
-      <c r="O48" s="54">
+      <c r="O48" s="57">
         <f>(1+O40)*(1-O44)/(1-N44)-1</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="14.4" customHeight="1">
-      <c r="B49" s="28" t="inlineStr">
+      <c r="B49" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J49" s="54">
+      <c r="J49" s="57">
         <f>(1+J41)*(1-J45)-1</f>
         <v/>
       </c>
-      <c r="K49" s="54">
+      <c r="K49" s="57">
         <f>(1+K41)*(1-K45)/(1-J45)-1</f>
         <v/>
       </c>
-      <c r="L49" s="54">
+      <c r="L49" s="57">
         <f>(1+L41)*(1-L45)/(1-K45)-1</f>
         <v/>
       </c>
-      <c r="M49" s="54">
+      <c r="M49" s="57">
         <f>(1+M41)*(1-M45)/(1-L45)-1</f>
         <v/>
       </c>
-      <c r="N49" s="54">
+      <c r="N49" s="57">
         <f>(1+N41)*(1-N45)/(1-M45)-1</f>
         <v/>
       </c>
-      <c r="O49" s="54">
+      <c r="O49" s="57">
         <f>(1+O41)*(1-O45)/(1-N45)-1</f>
         <v/>
       </c>
     </row>
     <row r="50" ht="14.4" customHeight="1"/>
     <row r="51" ht="14.4" customHeight="1">
-      <c r="B51" s="55" t="inlineStr">
+      <c r="B51" s="58" t="inlineStr">
         <is>
           <t>▸ DETAIL: subject rent source by year &amp; reconciliation (grouped — click − to collapse)</t>
         </is>
       </c>
     </row>
     <row r="52" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B52" s="57" t="inlineStr">
+      <c r="B52" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y6  Q3 2019–Q2 2020</t>
         </is>
       </c>
-      <c r="E52" s="57" t="inlineStr">
+      <c r="E52" s="60" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="53" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B53" s="57" t="inlineStr">
+      <c r="B53" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y5  Q3 2020–Q2 2021</t>
         </is>
       </c>
-      <c r="E53" s="57" t="inlineStr">
+      <c r="E53" s="60" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="54" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B54" s="57" t="inlineStr">
+      <c r="B54" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y4  Q3 2021–Q2 2022</t>
         </is>
       </c>
-      <c r="E54" s="57" t="inlineStr">
+      <c r="E54" s="60" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="55" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B55" s="57" t="inlineStr">
+      <c r="B55" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y3  Q3 2022–Q2 2023</t>
         </is>
       </c>
-      <c r="E55" s="57" t="inlineStr">
+      <c r="E55" s="60" t="inlineStr">
         <is>
           <t>RealPage</t>
         </is>
       </c>
     </row>
     <row r="56" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B56" s="57" t="inlineStr">
+      <c r="B56" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y2  Q3 2023–Q2 2024</t>
         </is>
       </c>
-      <c r="E56" s="57" t="inlineStr">
+      <c r="E56" s="60" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
     <row r="57" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B57" s="57" t="inlineStr">
+      <c r="B57" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y1  Q3 2024–Q2 2025</t>
         </is>
       </c>
-      <c r="E57" s="57" t="inlineStr">
+      <c r="E57" s="60" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
     <row r="58" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B58" s="57" t="inlineStr">
+      <c r="B58" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  Y0  Q3 2025–Q2 2026</t>
         </is>
       </c>
-      <c r="E58" s="57" t="inlineStr">
+      <c r="E58" s="60" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
     <row r="59" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B59" s="57" t="inlineStr">
+      <c r="B59" s="60" t="inlineStr">
         <is>
           <t xml:space="preserve">  UC scheduled vs CoStar UC</t>
         </is>
       </c>
-      <c r="E59" s="57" t="inlineStr">
+      <c r="E59" s="60" t="inlineStr">
         <is>
           <t>885 / 336</t>
         </is>
       </c>
     </row>
     <row r="60" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B60" s="26" t="inlineStr">
+      <c r="B60" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  As-of 2026 Q2 QTD is partial (QTD); occupancy is point-in-time, Y0 flow sums partial.</t>
         </is>
@@ -3077,62 +3117,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="61" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="B1" s="58" t="inlineStr">
+      <c r="B1" s="61" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="C1" s="58" t="inlineStr">
+      <c r="C1" s="61" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D1" s="58" t="inlineStr">
+      <c r="D1" s="61" t="inlineStr">
         <is>
           <t>Year Built</t>
         </is>
       </c>
-      <c r="E1" s="58" t="inlineStr">
+      <c r="E1" s="61" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="F1" s="58" t="inlineStr">
+      <c r="F1" s="61" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="G1" s="58" t="inlineStr">
+      <c r="G1" s="61" t="inlineStr">
         <is>
           <t>CoStar Occ</t>
         </is>
       </c>
-      <c r="H1" s="58" t="inlineStr">
+      <c r="H1" s="61" t="inlineStr">
         <is>
           <t>RealPage Occ</t>
         </is>
       </c>
-      <c r="I1" s="58" t="inlineStr">
+      <c r="I1" s="61" t="inlineStr">
         <is>
           <t>CoStar Ask Rent</t>
         </is>
       </c>
-      <c r="J1" s="58" t="inlineStr">
+      <c r="J1" s="61" t="inlineStr">
         <is>
           <t>RealPage Eff Rent</t>
         </is>
       </c>
-      <c r="K1" s="58" t="inlineStr">
+      <c r="K1" s="61" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="L1" s="58" t="inlineStr">
+      <c r="L1" s="61" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3165,16 +3205,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G2" s="59" t="n">
+      <c r="G2" s="62" t="n">
         <v>0.926316</v>
       </c>
-      <c r="H2" s="59" t="n">
+      <c r="H2" s="62" t="n">
         <v>0.953</v>
       </c>
-      <c r="I2" s="60" t="n">
+      <c r="I2" s="63" t="n">
         <v>1795</v>
       </c>
-      <c r="J2" s="60" t="n">
+      <c r="J2" s="63" t="n">
         <v>1709</v>
       </c>
       <c r="K2" t="inlineStr">
@@ -3215,16 +3255,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G3" s="59" t="n">
+      <c r="G3" s="62" t="n">
         <v>0.902778</v>
       </c>
-      <c r="H3" s="59" t="n">
+      <c r="H3" s="62" t="n">
         <v>0.95</v>
       </c>
-      <c r="I3" s="60" t="n">
+      <c r="I3" s="63" t="n">
         <v>1765</v>
       </c>
-      <c r="J3" s="60" t="n">
+      <c r="J3" s="63" t="n">
         <v>1793</v>
       </c>
       <c r="K3" t="inlineStr">
@@ -3265,16 +3305,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G4" s="59" t="n">
+      <c r="G4" s="62" t="n">
         <v>0.879365</v>
       </c>
-      <c r="H4" s="59" t="n">
+      <c r="H4" s="62" t="n">
         <v>0.911</v>
       </c>
-      <c r="I4" s="60" t="n">
+      <c r="I4" s="63" t="n">
         <v>1836</v>
       </c>
-      <c r="J4" s="60" t="n">
+      <c r="J4" s="63" t="n">
         <v>1821</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -3315,16 +3355,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G5" s="59" t="n">
+      <c r="G5" s="62" t="n">
         <v>0.92</v>
       </c>
-      <c r="H5" s="59" t="n">
+      <c r="H5" s="62" t="n">
         <v>0.929</v>
       </c>
-      <c r="I5" s="60" t="n">
+      <c r="I5" s="63" t="n">
         <v>1861</v>
       </c>
-      <c r="J5" s="60" t="n">
+      <c r="J5" s="63" t="n">
         <v>1439</v>
       </c>
       <c r="K5" t="inlineStr">
@@ -3365,16 +3405,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G6" s="59" t="n">
+      <c r="G6" s="62" t="n">
         <v>0.948454</v>
       </c>
-      <c r="H6" s="59" t="n">
+      <c r="H6" s="62" t="n">
         <v>0.952</v>
       </c>
-      <c r="I6" s="60" t="n">
+      <c r="I6" s="63" t="n">
         <v>1897</v>
       </c>
-      <c r="J6" s="60" t="n">
+      <c r="J6" s="63" t="n">
         <v>1927</v>
       </c>
       <c r="K6" t="inlineStr">
@@ -3411,10 +3451,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G7" s="59" t="n"/>
-      <c r="H7" s="59" t="n"/>
-      <c r="I7" s="60" t="n"/>
-      <c r="J7" s="60" t="n"/>
+      <c r="G7" s="62" t="n"/>
+      <c r="H7" s="62" t="n"/>
+      <c r="I7" s="63" t="n"/>
+      <c r="J7" s="63" t="n"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3453,10 +3493,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G8" s="59" t="n"/>
-      <c r="H8" s="59" t="n"/>
-      <c r="I8" s="60" t="n"/>
-      <c r="J8" s="60" t="n"/>
+      <c r="G8" s="62" t="n"/>
+      <c r="H8" s="62" t="n"/>
+      <c r="I8" s="63" t="n"/>
+      <c r="J8" s="63" t="n"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3495,10 +3535,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G9" s="59" t="n"/>
-      <c r="H9" s="59" t="n"/>
-      <c r="I9" s="60" t="n"/>
-      <c r="J9" s="60" t="n"/>
+      <c r="G9" s="62" t="n"/>
+      <c r="H9" s="62" t="n"/>
+      <c r="I9" s="63" t="n"/>
+      <c r="J9" s="63" t="n"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3537,10 +3577,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G10" s="59" t="n"/>
-      <c r="H10" s="59" t="n"/>
-      <c r="I10" s="60" t="n"/>
-      <c r="J10" s="60" t="n"/>
+      <c r="G10" s="62" t="n"/>
+      <c r="H10" s="62" t="n"/>
+      <c r="I10" s="63" t="n"/>
+      <c r="J10" s="63" t="n"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3579,10 +3619,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G11" s="59" t="n"/>
-      <c r="H11" s="59" t="n"/>
-      <c r="I11" s="60" t="n"/>
-      <c r="J11" s="60" t="n"/>
+      <c r="G11" s="62" t="n"/>
+      <c r="H11" s="62" t="n"/>
+      <c r="I11" s="63" t="n"/>
+      <c r="J11" s="63" t="n"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3621,10 +3661,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G12" s="59" t="n"/>
-      <c r="H12" s="59" t="n"/>
-      <c r="I12" s="60" t="n"/>
-      <c r="J12" s="60" t="n"/>
+      <c r="G12" s="62" t="n"/>
+      <c r="H12" s="62" t="n"/>
+      <c r="I12" s="63" t="n"/>
+      <c r="J12" s="63" t="n"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3655,10 +3695,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G13" s="59" t="n"/>
-      <c r="H13" s="59" t="n"/>
-      <c r="I13" s="60" t="n"/>
-      <c r="J13" s="60" t="n"/>
+      <c r="G13" s="62" t="n"/>
+      <c r="H13" s="62" t="n"/>
+      <c r="I13" s="63" t="n"/>
+      <c r="J13" s="63" t="n"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3689,10 +3729,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G14" s="59" t="n"/>
-      <c r="H14" s="59" t="n"/>
-      <c r="I14" s="60" t="n"/>
-      <c r="J14" s="60" t="n"/>
+      <c r="G14" s="62" t="n"/>
+      <c r="H14" s="62" t="n"/>
+      <c r="I14" s="63" t="n"/>
+      <c r="J14" s="63" t="n"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3723,10 +3763,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G15" s="59" t="n"/>
-      <c r="H15" s="59" t="n"/>
-      <c r="I15" s="60" t="n"/>
-      <c r="J15" s="60" t="n"/>
+      <c r="G15" s="62" t="n"/>
+      <c r="H15" s="62" t="n"/>
+      <c r="I15" s="63" t="n"/>
+      <c r="J15" s="63" t="n"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3757,10 +3797,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G16" s="59" t="n"/>
-      <c r="H16" s="59" t="n"/>
-      <c r="I16" s="60" t="n"/>
-      <c r="J16" s="60" t="n"/>
+      <c r="G16" s="62" t="n"/>
+      <c r="H16" s="62" t="n"/>
+      <c r="I16" s="63" t="n"/>
+      <c r="J16" s="63" t="n"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3797,494 +3837,494 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="61" t="inlineStr">
+      <c r="B2" s="64" t="inlineStr">
         <is>
           <t>PIPELINE DILIGENCE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="39" t="inlineStr">
+      <c r="B3" s="42" t="inlineStr">
         <is>
           <t>Property / Site</t>
         </is>
       </c>
-      <c r="C3" s="39" t="inlineStr">
+      <c r="C3" s="42" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D3" s="39" t="inlineStr">
+      <c r="D3" s="42" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="E3" s="39" t="inlineStr">
+      <c r="E3" s="42" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F3" s="39" t="inlineStr">
+      <c r="F3" s="42" t="inlineStr">
         <is>
           <t>Leasing Pace</t>
         </is>
       </c>
-      <c r="G3" s="39" t="inlineStr">
+      <c r="G3" s="42" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H3" s="39" t="inlineStr">
+      <c r="H3" s="42" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="32" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>Riverview at Clear Creek</t>
         </is>
       </c>
-      <c r="C4" s="62" t="inlineStr">
+      <c r="C4" s="65" t="inlineStr">
         <is>
           <t>298</t>
         </is>
       </c>
-      <c r="D4" s="62" t="n"/>
-      <c r="E4" s="32" t="inlineStr">
+      <c r="D4" s="65" t="n"/>
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F4" s="32" t="n"/>
-      <c r="G4" s="32" t="inlineStr">
+      <c r="F4" s="35" t="n"/>
+      <c r="G4" s="35" t="inlineStr">
         <is>
           <t>WB Property Group; waterfront mixed-use (marina/hotel/townhomes) incl senior-housing component; CoStar 'under construction' NOT corroborated, public record stalls ~2022-23; market-rate; full plan ~2029</t>
         </is>
       </c>
-      <c r="H4" s="32" t="inlineStr">
+      <c r="H4" s="35" t="inlineStr">
         <is>
           <t>https://communityimpact.com/houston/bay-area/development/2022/04/22/making-a-destination-league-city-developer-sign-agreement-to-build-riverview/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="32" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Lenox Clear Creek</t>
         </is>
       </c>
-      <c r="C5" s="62" t="inlineStr">
+      <c r="C5" s="65" t="inlineStr">
         <is>
           <t>336</t>
         </is>
       </c>
-      <c r="D5" s="62" t="inlineStr">
+      <c r="D5" s="65" t="inlineStr">
         <is>
           <t>Q3 2027</t>
         </is>
       </c>
-      <c r="E5" s="32" t="inlineStr">
+      <c r="E5" s="35" t="inlineStr">
         <is>
           <t>under construction</t>
         </is>
       </c>
-      <c r="F5" s="32" t="n"/>
-      <c r="G5" s="32" t="inlineStr">
+      <c r="F5" s="35" t="n"/>
+      <c r="G5" s="35" t="inlineStr">
         <is>
           <t>Likely CoStar placeholder = OHT Partners + Crow Holdings JV, 16200 SH-3; broke ground late 2025; market-rate; LOCATION is Clear Lake 77058 (~Webster), NOT League City - weaker overlap</t>
         </is>
       </c>
-      <c r="H5" s="32" t="inlineStr">
+      <c r="H5" s="35" t="inlineStr">
         <is>
           <t>https://rebusinessonline.com/oht-partners-crow-holdings-break-ground-on-336-unit-multifamily-project-in-metro-houston/</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="32" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Dakota at Kemah</t>
         </is>
       </c>
-      <c r="C6" s="62" t="inlineStr">
+      <c r="C6" s="65" t="inlineStr">
         <is>
           <t>229</t>
         </is>
       </c>
-      <c r="D6" s="62" t="inlineStr">
+      <c r="D6" s="65" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
       </c>
-      <c r="E6" s="32" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>under construction</t>
         </is>
       </c>
-      <c r="F6" s="32" t="n"/>
-      <c r="G6" s="32" t="inlineStr">
+      <c r="F6" s="35" t="n"/>
+      <c r="G6" s="35" t="inlineStr">
         <is>
           <t>Dakota Enterprises; mgmt The Mathis Group; 2801 Lawrence Rd Kemah; 10 three-story bldgs; groundbreaking Dec 9 2025; TDLR completion Jan 15 2027; market-rate luxury</t>
         </is>
       </c>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="35" t="inlineStr">
         <is>
           <t>https://communityimpact.com/houston/bay-area/government/2025/12/03/the-dakota-at-kemah-to-have-groundbreaking-ceremony/</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="32" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>The League I</t>
         </is>
       </c>
-      <c r="C7" s="62" t="inlineStr">
+      <c r="C7" s="65" t="inlineStr">
         <is>
           <t>304</t>
         </is>
       </c>
-      <c r="D7" s="62" t="inlineStr">
+      <c r="D7" s="65" t="inlineStr">
         <is>
           <t>Q3 2026</t>
         </is>
       </c>
-      <c r="E7" s="32" t="inlineStr">
+      <c r="E7" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F7" s="32" t="n"/>
-      <c r="G7" s="32" t="inlineStr">
+      <c r="F7" s="35" t="n"/>
+      <c r="G7" s="35" t="inlineStr">
         <is>
           <t>CJ Development (Johnny Vassallo); $125M 44-ac mixed-use FM-518; 304 Phase-1 count UNCONFIRMED (public sourcing ~600 total); no verified groundbreaking, prior multi-yr stall - field-verify vertical status</t>
         </is>
       </c>
-      <c r="H7" s="32" t="inlineStr">
+      <c r="H7" s="35" t="inlineStr">
         <is>
           <t>https://communityimpact.com/houston/bay-area/development/2026/03/31/new-modern-retail-dining-space-coming-to-league-city/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>The Edge at Seabrook Town Centre</t>
         </is>
       </c>
-      <c r="C8" s="62" t="inlineStr">
+      <c r="C8" s="65" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="D8" s="62" t="inlineStr">
+      <c r="D8" s="65" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
       </c>
-      <c r="E8" s="32" t="inlineStr">
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>under construction</t>
         </is>
       </c>
-      <c r="F8" s="32" t="n"/>
-      <c r="G8" s="32" t="inlineStr">
+      <c r="F8" s="35" t="n"/>
+      <c r="G8" s="35" t="inlineStr">
         <is>
           <t>HS Development Group; $85M 19.5-ac mixed-use; broke ground Jan 2026 after ~3-yr financing stall; 4-story garden + 28.5k sf retail; market-rate (rents $1.5k-$3.1k); buildout Q2 2028</t>
         </is>
       </c>
-      <c r="H8" s="32" t="inlineStr">
+      <c r="H8" s="35" t="inlineStr">
         <is>
           <t>https://therealdeal.com/texas/2026/01/16/hs-development-groups-seabrook-town-centre-breaks-ground/</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="32" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>The League Future Phases</t>
         </is>
       </c>
-      <c r="C9" s="62" t="inlineStr">
+      <c r="C9" s="65" t="inlineStr">
         <is>
           <t>400</t>
         </is>
       </c>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="32" t="inlineStr">
+      <c r="D9" s="65" t="n"/>
+      <c r="E9" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F9" s="32" t="n"/>
-      <c r="G9" s="32" t="inlineStr">
+      <c r="F9" s="35" t="n"/>
+      <c r="G9" s="35" t="inlineStr">
         <is>
           <t>CJ Development; future tranche of The League (FM-518); total project described up to ~600 units across phases so 400 future phase plausible but specific count NOT independently verified; market-rate</t>
         </is>
       </c>
-      <c r="H9" s="32" t="inlineStr">
+      <c r="H9" s="35" t="inlineStr">
         <is>
           <t>https://communityimpact.com/houston/bay-area/development/2022/01/27/45-acre-mixed-use-development-the-league-to-bring-retail-restaurants-homes-to-league-city/</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Residences at Highland Center</t>
         </is>
       </c>
-      <c r="C10" s="62" t="inlineStr">
+      <c r="C10" s="65" t="inlineStr">
         <is>
           <t>275</t>
         </is>
       </c>
-      <c r="D10" s="62" t="n"/>
-      <c r="E10" s="32" t="inlineStr">
+      <c r="D10" s="65" t="n"/>
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F10" s="32" t="n"/>
-      <c r="G10" s="32" t="inlineStr">
+      <c r="F10" s="35" t="n"/>
+      <c r="G10" s="35" t="inlineStr">
         <is>
           <t>UNVERIFIED - no public news, city agenda, or developer source found tying a ~275-unit MF project to Highland Center; possible CoStar/RealPage early-stage or speculative entry</t>
         </is>
       </c>
-      <c r="H10" s="32" t="inlineStr">
+      <c r="H10" s="35" t="inlineStr">
         <is>
           <t>not found</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="32" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Seabrook Plaza</t>
         </is>
       </c>
-      <c r="C11" s="62" t="inlineStr">
+      <c r="C11" s="65" t="inlineStr">
         <is>
           <t>260</t>
         </is>
       </c>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="32" t="inlineStr">
+      <c r="D11" s="65" t="n"/>
+      <c r="E11" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F11" s="32" t="n"/>
-      <c r="G11" s="32" t="inlineStr">
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="35" t="inlineStr">
         <is>
           <t>UNVERIFIED - could not confirm a 260-unit 'Seabrook Plaza' MF project; may be alias/duplicate of The Edge at Seabrook Town Centre or speculative CoStar entry</t>
         </is>
       </c>
-      <c r="H11" s="32" t="inlineStr">
+      <c r="H11" s="35" t="inlineStr">
         <is>
           <t>not found</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="32" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Avalon at Kemah I</t>
         </is>
       </c>
-      <c r="C12" s="62" t="inlineStr">
+      <c r="C12" s="65" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="D12" s="62" t="n"/>
-      <c r="E12" s="32" t="inlineStr">
+      <c r="D12" s="65" t="n"/>
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F12" s="32" t="n"/>
-      <c r="G12" s="32" t="inlineStr">
+      <c r="F12" s="35" t="n"/>
+      <c r="G12" s="35" t="inlineStr">
         <is>
           <t>UNVERIFIED - no public record of an 'Avalon at Kemah' apartment project; Kemah's only verified active MF is The Dakota; possible CoStar placeholder/rename</t>
         </is>
       </c>
-      <c r="H12" s="32" t="inlineStr">
+      <c r="H12" s="35" t="inlineStr">
         <is>
           <t>not found</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="32" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>Avalon at Kemah II</t>
         </is>
       </c>
-      <c r="C13" s="62" t="inlineStr">
+      <c r="C13" s="65" t="inlineStr">
         <is>
           <t>228</t>
         </is>
       </c>
-      <c r="D13" s="62" t="n"/>
-      <c r="E13" s="32" t="inlineStr">
+      <c r="D13" s="65" t="n"/>
+      <c r="E13" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="F13" s="32" t="n"/>
-      <c r="G13" s="32" t="inlineStr">
+      <c r="F13" s="35" t="n"/>
+      <c r="G13" s="35" t="inlineStr">
         <is>
           <t>UNVERIFIED - Phase II of an unverified Phase I; no public confirmation found; treat as speculative pending Kemah planning dept / CoStar source check</t>
         </is>
       </c>
-      <c r="H13" s="32" t="inlineStr">
+      <c r="H13" s="35" t="inlineStr">
         <is>
           <t>not found</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="61" t="inlineStr">
+      <c r="B15" s="64" t="inlineStr">
         <is>
           <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="39" t="inlineStr">
+      <c r="B16" s="42" t="inlineStr">
         <is>
           <t>Property / Site</t>
         </is>
       </c>
-      <c r="C16" s="39" t="inlineStr">
+      <c r="C16" s="42" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D16" s="39" t="inlineStr">
+      <c r="D16" s="42" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="E16" s="39" t="inlineStr">
+      <c r="E16" s="42" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="F16" s="39" t="inlineStr">
+      <c r="F16" s="42" t="inlineStr">
         <is>
           <t>Leasing Pace</t>
         </is>
       </c>
-      <c r="G16" s="39" t="inlineStr">
+      <c r="G16" s="42" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H16" s="39" t="inlineStr">
+      <c r="H16" s="42" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="32" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Westland Ranch MPC potential MF tract</t>
         </is>
       </c>
-      <c r="C17" s="62" t="n"/>
-      <c r="D17" s="62" t="n"/>
-      <c r="E17" s="32" t="inlineStr">
+      <c r="C17" s="65" t="n"/>
+      <c r="D17" s="65" t="n"/>
+      <c r="E17" s="35" t="inlineStr">
         <is>
           <t>planned/speculative</t>
         </is>
       </c>
-      <c r="F17" s="32" t="n"/>
-      <c r="G17" s="32" t="inlineStr">
+      <c r="F17" s="35" t="n"/>
+      <c r="G17" s="35" t="inlineStr">
         <is>
           <t>Meritage Homes MPC, W League City near SH-99/FM-517 (~5-6 mi, radius edge); ~1,200+ SF lots; no confirmed apartment phase but large MPCs often carry MF tracts; MF entitlement UNVERIFIED</t>
         </is>
       </c>
-      <c r="H17" s="32" t="inlineStr">
+      <c r="H17" s="35" t="inlineStr">
         <is>
           <t>https://www.meritagehomes.com/state/tx/houston/westland-ranch</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>FM-518 / Main St corridor mixed-use capacity</t>
         </is>
       </c>
-      <c r="C18" s="62" t="n"/>
-      <c r="D18" s="62" t="n"/>
-      <c r="E18" s="32" t="inlineStr">
+      <c r="C18" s="65" t="n"/>
+      <c r="D18" s="65" t="n"/>
+      <c r="E18" s="35" t="inlineStr">
         <is>
           <t>zoning/entitlement capacity</t>
         </is>
       </c>
-      <c r="F18" s="32" t="n"/>
-      <c r="G18" s="32" t="inlineStr">
+      <c r="F18" s="35" t="n"/>
+      <c r="G18" s="35" t="inlineStr">
         <is>
           <t>League City comp plan &amp; recent rezonings along FM-518 favor mixed-use w/ residential (The League sits here); latent MF capacity exists but no specific unnamed funded project confirmed</t>
         </is>
       </c>
-      <c r="H18" s="32" t="inlineStr">
+      <c r="H18" s="35" t="inlineStr">
         <is>
           <t>https://www.leaguecitytx.gov/151/Planning</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="32" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>Webster / SH-3 &amp; Bay Area Blvd MF node</t>
         </is>
       </c>
-      <c r="C19" s="62" t="n"/>
-      <c r="D19" s="62" t="n"/>
-      <c r="E19" s="32" t="inlineStr">
+      <c r="C19" s="65" t="n"/>
+      <c r="D19" s="65" t="n"/>
+      <c r="E19" s="35" t="inlineStr">
         <is>
           <t>redevelopment node</t>
         </is>
       </c>
-      <c r="F19" s="32" t="n"/>
-      <c r="G19" s="32" t="inlineStr">
+      <c r="F19" s="35" t="n"/>
+      <c r="G19" s="35" t="inlineStr">
         <is>
           <t>Webster (Baybrook/I-45 hub, ~4-5 mi N) actively courts MF; OHT/Crow 336u JV sits here; likely additional latent MF capacity but no specific unnamed verified project found</t>
         </is>
       </c>
-      <c r="H19" s="32" t="inlineStr">
+      <c r="H19" s="35" t="inlineStr">
         <is>
           <t>https://www.cityofwebster.com</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="32" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Friendswood multifamily</t>
         </is>
       </c>
-      <c r="C20" s="62" t="n"/>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="32" t="inlineStr">
+      <c r="C20" s="65" t="n"/>
+      <c r="D20" s="65" t="n"/>
+      <c r="E20" s="35" t="inlineStr">
         <is>
           <t>none confirmed</t>
         </is>
       </c>
-      <c r="F20" s="32" t="n"/>
-      <c r="G20" s="32" t="inlineStr">
+      <c r="F20" s="35" t="n"/>
+      <c r="G20" s="35" t="inlineStr">
         <is>
           <t>Friendswood largely SF-oriented, historically resistant to high-density MF; some mixed-use discussion at FM-518/FM-528 but nothing concrete; no specific latent apartment project found</t>
         </is>
       </c>
-      <c r="H20" s="32" t="inlineStr">
+      <c r="H20" s="35" t="inlineStr">
         <is>
           <t>not found</t>
         </is>

</xml_diff>

<commit_message>
Fix proximity geocoding, satellite map, brighter markers
- geo.Locator now retries with relaxed queries (drops the wrong-city
  component common in roster exports) and rejects any hit >8 mi from the
  subject before falling back to a ZIP centroid, so a mis-geocoded street
  name can no longer produce a wild distance. This corrects The Reserve at
  Baybrook (was a 7.2-mi ZIP-centroid artifact -> 5.4 mi, at the radius
  edge) without introducing the Lenox Bayside / "The League" far-match
  errors the naive relaxation caused.
- Map: default basemap is now satellite; saturated marker colours with
  white halos (Under Construction = visible spring green), yellow 5-mile
  ring, outlined labels for legibility over imagery.
- Regenerate all three example workbooks and the Aura satellite map.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="I7" s="12" t="n">
-        <v>7.2</v>
+        <v>5.4</v>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="I13" s="20" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="J13" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Make model-link the default and fill subject YoY/concession forward
The subject Market/Effective Rent and Occupancy rows now carry IFERROR'd
internal model links by default (Y0 falls back to the chart's own value,
Y1..Y6 to blank), so every chart is carry-over-ready and shows clean blanks
standalone instead of #REF. Pass --no-model-link for a pure standalone.

The subject YoY% and Concession% rows are now written for every column
(historical + forecast), not just history, so they populate once the rent
rows have data (the previously-blank forecast cells are the fix).

SKILL.md updated for the default flip and the drag/embed delivery modes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -2259,15 +2259,34 @@
       <c r="H23" s="48" t="n">
         <v>1793</v>
       </c>
-      <c r="I23" s="48" t="n">
-        <v>1782</v>
-      </c>
-      <c r="J23" s="49" t="n"/>
-      <c r="K23" s="49" t="n"/>
-      <c r="L23" s="49" t="n"/>
-      <c r="M23" s="49" t="n"/>
-      <c r="N23" s="49" t="n"/>
-      <c r="O23" s="49" t="n"/>
+      <c r="I23" s="48">
+        <f>IFERROR('Cash Flow (Annual)'!$F$4,1782)</f>
+        <v/>
+      </c>
+      <c r="J23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$K$4,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$L$4,"")</f>
+        <v/>
+      </c>
+      <c r="L23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$M$4,"")</f>
+        <v/>
+      </c>
+      <c r="M23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$N$4,"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$O$4,"")</f>
+        <v/>
+      </c>
+      <c r="O23" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$P$4,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24" ht="14.4" customHeight="1">
       <c r="B24" s="50" t="inlineStr">
@@ -2300,12 +2319,30 @@
         <f>IFERROR(I23/H23-1,"")</f>
         <v/>
       </c>
-      <c r="J24" s="52" t="n"/>
-      <c r="K24" s="52" t="n"/>
-      <c r="L24" s="52" t="n"/>
-      <c r="M24" s="52" t="n"/>
-      <c r="N24" s="52" t="n"/>
-      <c r="O24" s="52" t="n"/>
+      <c r="J24" s="52">
+        <f>IFERROR(J23/I23-1,"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="52">
+        <f>IFERROR(K23/J23-1,"")</f>
+        <v/>
+      </c>
+      <c r="L24" s="52">
+        <f>IFERROR(L23/K23-1,"")</f>
+        <v/>
+      </c>
+      <c r="M24" s="52">
+        <f>IFERROR(M23/L23-1,"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="52">
+        <f>IFERROR(N23/M23-1,"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="52">
+        <f>IFERROR(O23/N23-1,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" ht="14.4" customHeight="1">
       <c r="B25" s="31" t="inlineStr">
@@ -2325,15 +2362,34 @@
       <c r="H25" s="48" t="n">
         <v>1697</v>
       </c>
-      <c r="I25" s="48" t="n">
-        <v>1543</v>
-      </c>
-      <c r="J25" s="49" t="n"/>
-      <c r="K25" s="49" t="n"/>
-      <c r="L25" s="49" t="n"/>
-      <c r="M25" s="49" t="n"/>
-      <c r="N25" s="49" t="n"/>
-      <c r="O25" s="49" t="n"/>
+      <c r="I25" s="48">
+        <f>IFERROR('Cash Flow (Annual)'!$F$5,1543)</f>
+        <v/>
+      </c>
+      <c r="J25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$K$5,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$L$5,"")</f>
+        <v/>
+      </c>
+      <c r="L25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$M$5,"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$N$5,"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$O$5,"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="49">
+        <f>IFERROR('Cash Flow (Annual)'!$P$5,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" ht="14.4" customHeight="1">
       <c r="B26" s="50" t="inlineStr">
@@ -2366,12 +2422,30 @@
         <f>IFERROR(I25/H25-1,"")</f>
         <v/>
       </c>
-      <c r="J26" s="52" t="n"/>
-      <c r="K26" s="52" t="n"/>
-      <c r="L26" s="52" t="n"/>
-      <c r="M26" s="52" t="n"/>
-      <c r="N26" s="52" t="n"/>
-      <c r="O26" s="52" t="n"/>
+      <c r="J26" s="52">
+        <f>IFERROR(J25/I25-1,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="52">
+        <f>IFERROR(K25/J25-1,"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="52">
+        <f>IFERROR(L25/K25-1,"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="52">
+        <f>IFERROR(M25/L25-1,"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="52">
+        <f>IFERROR(N25/M25-1,"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="52">
+        <f>IFERROR(O25/N25-1,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="14.4" customHeight="1">
       <c r="B27" s="31" t="inlineStr">
@@ -2391,15 +2465,34 @@
       <c r="H27" s="53" t="n">
         <v>0.9324033975977525</v>
       </c>
-      <c r="I27" s="53" t="n">
-        <v>0.9194867500515453</v>
-      </c>
-      <c r="J27" s="54" t="n"/>
-      <c r="K27" s="54" t="n"/>
-      <c r="L27" s="54" t="n"/>
-      <c r="M27" s="54" t="n"/>
-      <c r="N27" s="54" t="n"/>
-      <c r="O27" s="54" t="n"/>
+      <c r="I27" s="53">
+        <f>IFERROR('Cash Flow (Annual)'!$F$14,0.9194867500515453)</f>
+        <v/>
+      </c>
+      <c r="J27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$K$14,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$L$14,"")</f>
+        <v/>
+      </c>
+      <c r="L27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$M$14,"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$N$14,"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$O$14,"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="54">
+        <f>IFERROR('Cash Flow (Annual)'!$P$14,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" ht="14.4" customHeight="1">
       <c r="B28" s="31" t="inlineStr">
@@ -2407,9 +2500,18 @@
           <t xml:space="preserve">  Concession %</t>
         </is>
       </c>
-      <c r="C28" s="53" t="n"/>
-      <c r="D28" s="53" t="n"/>
-      <c r="E28" s="53" t="n"/>
+      <c r="C28" s="53">
+        <f>IFERROR((C23-C25)/C23,"")</f>
+        <v/>
+      </c>
+      <c r="D28" s="53">
+        <f>IFERROR((D23-D25)/D23,"")</f>
+        <v/>
+      </c>
+      <c r="E28" s="53">
+        <f>IFERROR((E23-E25)/E23,"")</f>
+        <v/>
+      </c>
       <c r="F28" s="53">
         <f>IFERROR((F23-F25)/F23,"")</f>
         <v/>
@@ -2426,12 +2528,30 @@
         <f>IFERROR((I23-I25)/I23,"")</f>
         <v/>
       </c>
-      <c r="J28" s="54" t="n"/>
-      <c r="K28" s="54" t="n"/>
-      <c r="L28" s="54" t="n"/>
-      <c r="M28" s="54" t="n"/>
-      <c r="N28" s="54" t="n"/>
-      <c r="O28" s="54" t="n"/>
+      <c r="J28" s="54">
+        <f>IFERROR((J23-J25)/J23,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="54">
+        <f>IFERROR((K23-K25)/K23,"")</f>
+        <v/>
+      </c>
+      <c r="L28" s="54">
+        <f>IFERROR((L23-L25)/L23,"")</f>
+        <v/>
+      </c>
+      <c r="M28" s="54">
+        <f>IFERROR((M23-M25)/M23,"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="54">
+        <f>IFERROR((N23-N25)/N23,"")</f>
+        <v/>
+      </c>
+      <c r="O28" s="54">
+        <f>IFERROR((O23-O25)/O23,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" ht="14.4" customHeight="1"/>
     <row r="30" hidden="1" ht="14.4" customHeight="1">

</xml_diff>

<commit_message>
Roster Avg Mkt Rent shows asking rent, never RealPage effective
Column G is a market/asking figure, but with --rent-source realpage it was
showing RealPage *effective* rent. RealPage's export carries only effective
rent, so it must not feed an asking column. Add a distinct asking_rent
(CoStar asking primary; RealPage asking only if its pull carries that column;
'average' blends available asking values) and use it for the roster column
and the map popup. RealPage effective is retained for the divergence note /
Reconciliation Log. --rent-source gains an 'average' choice.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -846,7 +846,7 @@
         <v>0.929</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1439</v>
+        <v>1861</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
         <v>0.952</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>1927</v>
+        <v>1897</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
         <v>0.911</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>1821</v>
+        <v>1836</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
         <v>0.95</v>
       </c>
       <c r="G9" s="11" t="n">
-        <v>1793</v>
+        <v>1765</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         <v>0.953</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>1709</v>
+        <v>1795</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 3rd-party forecast block, collapse scenario inputs, align to model
Supply & Absorption tab now carries a model-linked "MARKET-RENT GROWTH —
TMG vs 3RD-PARTY FORECAST" block: CoStar/RealPage/Yardi/GreenStreet growth
from the model's 'Rent & Occ Data' (rows 31-34), a 4-source consensus, and
TMG's own growth (the gold focus row), each with a per-row AVG. Resolves
when the tab is carried into the model.

The Bear/Base/Bull scenario machinery (implied occupancy, market-rent-growth
& concession assumptions, derived effective-rent growth) is collapsed under a
single summary header so the tab leads with the supply/occupancy story and
the TMG-vs-forecast read.

Formatting aligned to the TMG model: navy FF153D64 section headers, blue-font
editable inputs (FF0000FF) on a light fill.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FFwLwTedaJX2Ztv3TDjAgH
</commit_message>
<xml_diff>
--- a/output/Aura_Beacon_Island__Supply_Chart.xlsx
+++ b/output/Aura_Beacon_Island__Supply_Chart.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="166" formatCode="0.0&quot; mi&quot;;;&quot;—&quot;"/>
     <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +75,19 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="FF0000FF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -88,6 +99,18 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="FF808080"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF153D64"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF595959"/>
       <sz val="8"/>
     </font>
     <font>
@@ -108,7 +131,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -117,7 +140,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1F3864"/>
+        <fgColor rgb="FF153D64"/>
       </patternFill>
     </fill>
     <fill>
@@ -165,6 +188,16 @@
         <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -192,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -278,10 +311,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -293,16 +326,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -329,11 +362,11 @@
     <xf numFmtId="167" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -345,23 +378,37 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1493,7 +1540,7 @@
     <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:Z60"/>
+  <dimension ref="B1:Z69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1511,6 +1558,7 @@
     <col width="9.5" customWidth="1" min="13" max="13"/>
     <col width="9.5" customWidth="1" min="14" max="14"/>
     <col width="9.5" customWidth="1" min="15" max="15"/>
+    <col width="9.5" customWidth="1" min="16" max="16"/>
     <col width="28" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
     <col width="11" customWidth="1" min="20" max="20"/>
@@ -2660,543 +2708,852 @@
     </row>
     <row r="32" ht="14.4" customHeight="1"/>
     <row r="33" ht="14.4" customHeight="1">
-      <c r="B33" s="31" t="inlineStr">
+      <c r="B33" s="30" t="inlineStr">
+        <is>
+          <t>MARKET-RENT GROWTH — TMG vs 3RD-PARTY FORECAST</t>
+        </is>
+      </c>
+      <c r="C33" s="56" t="n"/>
+      <c r="D33" s="56" t="n"/>
+      <c r="E33" s="56" t="n"/>
+      <c r="F33" s="56" t="n"/>
+      <c r="G33" s="56" t="n"/>
+      <c r="H33" s="56" t="n"/>
+      <c r="I33" s="56" t="n"/>
+      <c r="J33" s="57" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="K33" s="57" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="L33" s="57" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+      <c r="M33" s="57" t="inlineStr">
+        <is>
+          <t>Y4</t>
+        </is>
+      </c>
+      <c r="N33" s="57" t="inlineStr">
+        <is>
+          <t>Y5</t>
+        </is>
+      </c>
+      <c r="O33" s="57" t="inlineStr">
+        <is>
+          <t>Y6</t>
+        </is>
+      </c>
+      <c r="P33" s="57" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="14.4" customHeight="1">
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CoStar</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="n"/>
+      <c r="D34" s="59" t="n"/>
+      <c r="E34" s="59" t="n"/>
+      <c r="F34" s="59" t="n"/>
+      <c r="G34" s="59" t="n"/>
+      <c r="H34" s="59" t="n"/>
+      <c r="I34" s="59" t="n"/>
+      <c r="J34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$C$31,"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$D$31,"")</f>
+        <v/>
+      </c>
+      <c r="L34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$E$31,"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$F$31,"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$G$31,"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$H$31,"")</f>
+        <v/>
+      </c>
+      <c r="P34" s="53">
+        <f>IFERROR(AVERAGE(J34:O34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="14.4" customHeight="1">
+      <c r="B35" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  RealPage</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="n"/>
+      <c r="D35" s="59" t="n"/>
+      <c r="E35" s="59" t="n"/>
+      <c r="F35" s="59" t="n"/>
+      <c r="G35" s="59" t="n"/>
+      <c r="H35" s="59" t="n"/>
+      <c r="I35" s="59" t="n"/>
+      <c r="J35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$C$32,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$D$32,"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$E$32,"")</f>
+        <v/>
+      </c>
+      <c r="M35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$F$32,"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$G$32,"")</f>
+        <v/>
+      </c>
+      <c r="O35" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$H$32,"")</f>
+        <v/>
+      </c>
+      <c r="P35" s="53">
+        <f>IFERROR(AVERAGE(J35:O35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="14.4" customHeight="1">
+      <c r="B36" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Yardi</t>
+        </is>
+      </c>
+      <c r="C36" s="59" t="n"/>
+      <c r="D36" s="59" t="n"/>
+      <c r="E36" s="59" t="n"/>
+      <c r="F36" s="59" t="n"/>
+      <c r="G36" s="59" t="n"/>
+      <c r="H36" s="59" t="n"/>
+      <c r="I36" s="59" t="n"/>
+      <c r="J36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$C$33,"")</f>
+        <v/>
+      </c>
+      <c r="K36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$D$33,"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$E$33,"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$F$33,"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$G$33,"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$H$33,"")</f>
+        <v/>
+      </c>
+      <c r="P36" s="53">
+        <f>IFERROR(AVERAGE(J36:O36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="14.4" customHeight="1">
+      <c r="B37" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  GreenStreet</t>
+        </is>
+      </c>
+      <c r="C37" s="59" t="n"/>
+      <c r="D37" s="59" t="n"/>
+      <c r="E37" s="59" t="n"/>
+      <c r="F37" s="59" t="n"/>
+      <c r="G37" s="59" t="n"/>
+      <c r="H37" s="59" t="n"/>
+      <c r="I37" s="59" t="n"/>
+      <c r="J37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$C$34,"")</f>
+        <v/>
+      </c>
+      <c r="K37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$D$34,"")</f>
+        <v/>
+      </c>
+      <c r="L37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$E$34,"")</f>
+        <v/>
+      </c>
+      <c r="M37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$F$34,"")</f>
+        <v/>
+      </c>
+      <c r="N37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$G$34,"")</f>
+        <v/>
+      </c>
+      <c r="O37" s="53">
+        <f>IFERROR('Rent &amp; Occ Data'!$H$34,"")</f>
+        <v/>
+      </c>
+      <c r="P37" s="53">
+        <f>IFERROR(AVERAGE(J37:O37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="14.4" customHeight="1">
+      <c r="B38" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Consensus (4-source avg)</t>
+        </is>
+      </c>
+      <c r="C38" s="61" t="n"/>
+      <c r="D38" s="61" t="n"/>
+      <c r="E38" s="61" t="n"/>
+      <c r="F38" s="61" t="n"/>
+      <c r="G38" s="61" t="n"/>
+      <c r="H38" s="61" t="n"/>
+      <c r="I38" s="61" t="n"/>
+      <c r="J38" s="62">
+        <f>IFERROR(AVERAGE(J34:J37),"")</f>
+        <v/>
+      </c>
+      <c r="K38" s="62">
+        <f>IFERROR(AVERAGE(K34:K37),"")</f>
+        <v/>
+      </c>
+      <c r="L38" s="62">
+        <f>IFERROR(AVERAGE(L34:L37),"")</f>
+        <v/>
+      </c>
+      <c r="M38" s="62">
+        <f>IFERROR(AVERAGE(M34:M37),"")</f>
+        <v/>
+      </c>
+      <c r="N38" s="62">
+        <f>IFERROR(AVERAGE(N34:N37),"")</f>
+        <v/>
+      </c>
+      <c r="O38" s="62">
+        <f>IFERROR(AVERAGE(O34:O37),"")</f>
+        <v/>
+      </c>
+      <c r="P38" s="62">
+        <f>IFERROR(AVERAGE(P34:P37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="14.4" customHeight="1">
+      <c r="B39" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  TMG — our market-rent growth  ◄</t>
+        </is>
+      </c>
+      <c r="C39" s="64" t="n"/>
+      <c r="D39" s="64" t="n"/>
+      <c r="E39" s="64" t="n"/>
+      <c r="F39" s="64" t="n"/>
+      <c r="G39" s="64" t="n"/>
+      <c r="H39" s="64" t="n"/>
+      <c r="I39" s="64" t="n"/>
+      <c r="J39" s="65">
+        <f>IFERROR(J24,"")</f>
+        <v/>
+      </c>
+      <c r="K39" s="65">
+        <f>IFERROR(K24,"")</f>
+        <v/>
+      </c>
+      <c r="L39" s="65">
+        <f>IFERROR(L24,"")</f>
+        <v/>
+      </c>
+      <c r="M39" s="65">
+        <f>IFERROR(M24,"")</f>
+        <v/>
+      </c>
+      <c r="N39" s="65">
+        <f>IFERROR(N24,"")</f>
+        <v/>
+      </c>
+      <c r="O39" s="65">
+        <f>IFERROR(O24,"")</f>
+        <v/>
+      </c>
+      <c r="P39" s="65">
+        <f>IFERROR(AVERAGE(J39:O39),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="14.4" customHeight="1"/>
+    <row r="41" ht="14.4" customHeight="1">
+      <c r="B41" s="66" t="inlineStr">
+        <is>
+          <t>▸ SCENARIO INPUTS — Bear / Base / Bull  (implied occupancy, rent-growth &amp; concession assumptions — click + to expand)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B42" s="31" t="inlineStr">
         <is>
           <t>IMPLIED 5-MI OCCUPANCY BY DEMAND SCENARIO</t>
         </is>
       </c>
-      <c r="J33" s="56" t="inlineStr">
+      <c r="J42" s="67" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K33" s="56" t="inlineStr">
+      <c r="K42" s="67" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L33" s="56" t="inlineStr">
+      <c r="L42" s="67" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M33" s="56" t="inlineStr">
+      <c r="M42" s="67" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N33" s="56" t="inlineStr">
+      <c r="N42" s="67" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O33" s="56" t="inlineStr">
+      <c r="O42" s="67" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="14.4" customHeight="1">
-      <c r="B34" s="31" t="inlineStr">
+    <row r="43" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B43" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J34" s="57">
+      <c r="J43" s="68">
         <f>MIN($C$6,($I$31+$C$8*1)/J30)</f>
         <v/>
       </c>
-      <c r="K34" s="57">
+      <c r="K43" s="68">
         <f>MIN($C$6,($I$31+$C$8*2)/K30)</f>
         <v/>
       </c>
-      <c r="L34" s="57">
+      <c r="L43" s="68">
         <f>MIN($C$6,($I$31+$C$8*3)/L30)</f>
         <v/>
       </c>
-      <c r="M34" s="57">
+      <c r="M43" s="68">
         <f>MIN($C$6,($I$31+$C$8*4)/M30)</f>
         <v/>
       </c>
-      <c r="N34" s="57">
+      <c r="N43" s="68">
         <f>MIN($C$6,($I$31+$C$8*5)/N30)</f>
         <v/>
       </c>
-      <c r="O34" s="57">
+      <c r="O43" s="68">
         <f>MIN($C$6,($I$31+$C$8*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="14.4" customHeight="1">
-      <c r="B35" s="31" t="inlineStr">
+    <row r="44" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B44" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J35" s="57">
+      <c r="J44" s="68">
         <f>MIN($C$6,($I$31+$C$9*1)/J30)</f>
         <v/>
       </c>
-      <c r="K35" s="57">
+      <c r="K44" s="68">
         <f>MIN($C$6,($I$31+$C$9*2)/K30)</f>
         <v/>
       </c>
-      <c r="L35" s="57">
+      <c r="L44" s="68">
         <f>MIN($C$6,($I$31+$C$9*3)/L30)</f>
         <v/>
       </c>
-      <c r="M35" s="57">
+      <c r="M44" s="68">
         <f>MIN($C$6,($I$31+$C$9*4)/M30)</f>
         <v/>
       </c>
-      <c r="N35" s="57">
+      <c r="N44" s="68">
         <f>MIN($C$6,($I$31+$C$9*5)/N30)</f>
         <v/>
       </c>
-      <c r="O35" s="57">
+      <c r="O44" s="68">
         <f>MIN($C$6,($I$31+$C$9*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="14.4" customHeight="1">
-      <c r="B36" s="31" t="inlineStr">
+    <row r="45" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B45" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J36" s="57">
+      <c r="J45" s="68">
         <f>MIN($C$6,($I$31+$C$10*1)/J30)</f>
         <v/>
       </c>
-      <c r="K36" s="57">
+      <c r="K45" s="68">
         <f>MIN($C$6,($I$31+$C$10*2)/K30)</f>
         <v/>
       </c>
-      <c r="L36" s="57">
+      <c r="L45" s="68">
         <f>MIN($C$6,($I$31+$C$10*3)/L30)</f>
         <v/>
       </c>
-      <c r="M36" s="57">
+      <c r="M45" s="68">
         <f>MIN($C$6,($I$31+$C$10*4)/M30)</f>
         <v/>
       </c>
-      <c r="N36" s="57">
+      <c r="N45" s="68">
         <f>MIN($C$6,($I$31+$C$10*5)/N30)</f>
         <v/>
       </c>
-      <c r="O36" s="57">
+      <c r="O45" s="68">
         <f>MIN($C$6,($I$31+$C$10*6)/O30)</f>
         <v/>
       </c>
     </row>
-    <row r="37" ht="14.4" customHeight="1"/>
-    <row r="38" ht="14.4" customHeight="1">
-      <c r="B38" s="31" t="inlineStr">
+    <row r="46" hidden="1" outlineLevel="1" ht="14.4" customHeight="1"/>
+    <row r="47" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B47" s="31" t="inlineStr">
         <is>
           <t>MARKET RENT GROWTH (editable assumptions)</t>
         </is>
       </c>
-      <c r="J38" s="58" t="inlineStr">
+      <c r="J47" s="69" t="inlineStr">
         <is>
           <t>Y1</t>
         </is>
       </c>
-      <c r="K38" s="58" t="inlineStr">
+      <c r="K47" s="69" t="inlineStr">
         <is>
           <t>Y2</t>
         </is>
       </c>
-      <c r="L38" s="58" t="inlineStr">
+      <c r="L47" s="69" t="inlineStr">
         <is>
           <t>Y3</t>
         </is>
       </c>
-      <c r="M38" s="58" t="inlineStr">
+      <c r="M47" s="69" t="inlineStr">
         <is>
           <t>Y4</t>
         </is>
       </c>
-      <c r="N38" s="58" t="inlineStr">
+      <c r="N47" s="69" t="inlineStr">
         <is>
           <t>Y5</t>
         </is>
       </c>
-      <c r="O38" s="58" t="inlineStr">
+      <c r="O47" s="69" t="inlineStr">
         <is>
           <t>Y6</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="14.4" customHeight="1">
-      <c r="B39" s="31" t="inlineStr">
+    <row r="48" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B48" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J39" s="59" t="n">
+      <c r="J48" s="70" t="n">
         <v>-0.0025</v>
       </c>
-      <c r="K39" s="59" t="n">
+      <c r="K48" s="70" t="n">
         <v>0.0175</v>
       </c>
-      <c r="L39" s="59" t="n">
+      <c r="L48" s="70" t="n">
         <v>0.0275</v>
       </c>
-      <c r="M39" s="59" t="n">
+      <c r="M48" s="70" t="n">
         <v>0.0375</v>
       </c>
-      <c r="N39" s="59" t="n">
+      <c r="N48" s="70" t="n">
         <v>0.0275</v>
       </c>
-      <c r="O39" s="59" t="n">
+      <c r="O48" s="70" t="n">
         <v>0.0175</v>
       </c>
     </row>
-    <row r="40" ht="14.4" customHeight="1">
-      <c r="B40" s="31" t="inlineStr">
+    <row r="49" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B49" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J40" s="59" t="n">
+      <c r="J49" s="70" t="n">
         <v>0.01</v>
       </c>
-      <c r="K40" s="59" t="n">
+      <c r="K49" s="70" t="n">
         <v>0.03</v>
       </c>
-      <c r="L40" s="59" t="n">
+      <c r="L49" s="70" t="n">
         <v>0.04</v>
       </c>
-      <c r="M40" s="59" t="n">
+      <c r="M49" s="70" t="n">
         <v>0.05</v>
       </c>
-      <c r="N40" s="59" t="n">
+      <c r="N49" s="70" t="n">
         <v>0.04</v>
       </c>
-      <c r="O40" s="59" t="n">
+      <c r="O49" s="70" t="n">
         <v>0.03</v>
       </c>
     </row>
-    <row r="41" ht="14.4" customHeight="1">
-      <c r="B41" s="31" t="inlineStr">
+    <row r="50" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B50" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J41" s="59" t="n">
+      <c r="J50" s="70" t="n">
         <v>0.02</v>
       </c>
-      <c r="K41" s="59" t="n">
+      <c r="K50" s="70" t="n">
         <v>0.04</v>
       </c>
-      <c r="L41" s="59" t="n">
+      <c r="L50" s="70" t="n">
         <v>0.05</v>
       </c>
-      <c r="M41" s="59" t="n">
+      <c r="M50" s="70" t="n">
         <v>0.06</v>
       </c>
-      <c r="N41" s="59" t="n">
+      <c r="N50" s="70" t="n">
         <v>0.05</v>
       </c>
-      <c r="O41" s="59" t="n">
+      <c r="O50" s="70" t="n">
         <v>0.04</v>
       </c>
     </row>
-    <row r="42" ht="14.4" customHeight="1">
-      <c r="B42" s="31" t="inlineStr">
+    <row r="51" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B51" s="31" t="inlineStr">
         <is>
           <t>CONCESSIONS % — forward assumption (editable)</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="14.4" customHeight="1">
-      <c r="B43" s="31" t="inlineStr">
+    <row r="52" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B52" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J43" s="59" t="n">
+      <c r="J52" s="70" t="n">
         <v>0.06</v>
       </c>
-      <c r="K43" s="59" t="n">
+      <c r="K52" s="70" t="n">
         <v>0.045</v>
       </c>
-      <c r="L43" s="59" t="n">
+      <c r="L52" s="70" t="n">
         <v>0.035</v>
       </c>
-      <c r="M43" s="59" t="n">
+      <c r="M52" s="70" t="n">
         <v>0.035</v>
       </c>
-      <c r="N43" s="59" t="n">
+      <c r="N52" s="70" t="n">
         <v>0.035</v>
       </c>
-      <c r="O43" s="59" t="n">
+      <c r="O52" s="70" t="n">
         <v>0.035</v>
       </c>
     </row>
-    <row r="44" ht="14.4" customHeight="1">
-      <c r="B44" s="31" t="inlineStr">
+    <row r="53" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B53" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J44" s="59" t="n">
+      <c r="J53" s="70" t="n">
         <v>0.03</v>
       </c>
-      <c r="K44" s="59" t="n">
+      <c r="K53" s="70" t="n">
         <v>0.015</v>
       </c>
-      <c r="L44" s="59" t="n">
+      <c r="L53" s="70" t="n">
         <v>0.005</v>
       </c>
-      <c r="M44" s="59" t="n">
+      <c r="M53" s="70" t="n">
         <v>0.005</v>
       </c>
-      <c r="N44" s="59" t="n">
+      <c r="N53" s="70" t="n">
         <v>0.005</v>
       </c>
-      <c r="O44" s="59" t="n">
+      <c r="O53" s="70" t="n">
         <v>0.005</v>
       </c>
     </row>
-    <row r="45" ht="14.4" customHeight="1">
-      <c r="B45" s="31" t="inlineStr">
+    <row r="54" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B54" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J45" s="59" t="n">
+      <c r="J54" s="70" t="n">
         <v>0.02</v>
       </c>
-      <c r="K45" s="59" t="n">
+      <c r="K54" s="70" t="n">
         <v>0.005</v>
       </c>
-      <c r="L45" s="59" t="n">
+      <c r="L54" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="M45" s="59" t="n">
+      <c r="M54" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="59" t="n">
+      <c r="N54" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="O45" s="59" t="n">
+      <c r="O54" s="70" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="14.4" customHeight="1">
-      <c r="B46" s="31" t="inlineStr">
+    <row r="55" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B55" s="31" t="inlineStr">
         <is>
           <t>EFFECTIVE RENT GROWTH (derived)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="14.4" customHeight="1">
-      <c r="B47" s="31" t="inlineStr">
+    <row r="56" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B56" s="31" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="J47" s="57">
-        <f>(1+J39)*(1-J43)-1</f>
-        <v/>
-      </c>
-      <c r="K47" s="57">
-        <f>(1+K39)*(1-K43)/(1-J43)-1</f>
-        <v/>
-      </c>
-      <c r="L47" s="57">
-        <f>(1+L39)*(1-L43)/(1-K43)-1</f>
-        <v/>
-      </c>
-      <c r="M47" s="57">
-        <f>(1+M39)*(1-M43)/(1-L43)-1</f>
-        <v/>
-      </c>
-      <c r="N47" s="57">
-        <f>(1+N39)*(1-N43)/(1-M43)-1</f>
-        <v/>
-      </c>
-      <c r="O47" s="57">
-        <f>(1+O39)*(1-O43)/(1-N43)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" ht="14.4" customHeight="1">
-      <c r="B48" s="31" t="inlineStr">
+      <c r="J56" s="68">
+        <f>(1+J48)*(1-J52)-1</f>
+        <v/>
+      </c>
+      <c r="K56" s="68">
+        <f>(1+K48)*(1-K52)/(1-J52)-1</f>
+        <v/>
+      </c>
+      <c r="L56" s="68">
+        <f>(1+L48)*(1-L52)/(1-K52)-1</f>
+        <v/>
+      </c>
+      <c r="M56" s="68">
+        <f>(1+M48)*(1-M52)/(1-L52)-1</f>
+        <v/>
+      </c>
+      <c r="N56" s="68">
+        <f>(1+N48)*(1-N52)/(1-M52)-1</f>
+        <v/>
+      </c>
+      <c r="O56" s="68">
+        <f>(1+O48)*(1-O52)/(1-N52)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B57" s="31" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="J48" s="57">
-        <f>(1+J40)*(1-J44)-1</f>
-        <v/>
-      </c>
-      <c r="K48" s="57">
-        <f>(1+K40)*(1-K44)/(1-J44)-1</f>
-        <v/>
-      </c>
-      <c r="L48" s="57">
-        <f>(1+L40)*(1-L44)/(1-K44)-1</f>
-        <v/>
-      </c>
-      <c r="M48" s="57">
-        <f>(1+M40)*(1-M44)/(1-L44)-1</f>
-        <v/>
-      </c>
-      <c r="N48" s="57">
-        <f>(1+N40)*(1-N44)/(1-M44)-1</f>
-        <v/>
-      </c>
-      <c r="O48" s="57">
-        <f>(1+O40)*(1-O44)/(1-N44)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" ht="14.4" customHeight="1">
-      <c r="B49" s="31" t="inlineStr">
+      <c r="J57" s="68">
+        <f>(1+J49)*(1-J53)-1</f>
+        <v/>
+      </c>
+      <c r="K57" s="68">
+        <f>(1+K49)*(1-K53)/(1-J53)-1</f>
+        <v/>
+      </c>
+      <c r="L57" s="68">
+        <f>(1+L49)*(1-L53)/(1-K53)-1</f>
+        <v/>
+      </c>
+      <c r="M57" s="68">
+        <f>(1+M49)*(1-M53)/(1-L53)-1</f>
+        <v/>
+      </c>
+      <c r="N57" s="68">
+        <f>(1+N49)*(1-N53)/(1-M53)-1</f>
+        <v/>
+      </c>
+      <c r="O57" s="68">
+        <f>(1+O49)*(1-O53)/(1-N53)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B58" s="31" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="J49" s="57">
-        <f>(1+J41)*(1-J45)-1</f>
-        <v/>
-      </c>
-      <c r="K49" s="57">
-        <f>(1+K41)*(1-K45)/(1-J45)-1</f>
-        <v/>
-      </c>
-      <c r="L49" s="57">
-        <f>(1+L41)*(1-L45)/(1-K45)-1</f>
-        <v/>
-      </c>
-      <c r="M49" s="57">
-        <f>(1+M41)*(1-M45)/(1-L45)-1</f>
-        <v/>
-      </c>
-      <c r="N49" s="57">
-        <f>(1+N41)*(1-N45)/(1-M45)-1</f>
-        <v/>
-      </c>
-      <c r="O49" s="57">
-        <f>(1+O41)*(1-O45)/(1-N45)-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="14.4" customHeight="1"/>
-    <row r="51" ht="14.4" customHeight="1">
-      <c r="B51" s="58" t="inlineStr">
+      <c r="J58" s="68">
+        <f>(1+J50)*(1-J54)-1</f>
+        <v/>
+      </c>
+      <c r="K58" s="68">
+        <f>(1+K50)*(1-K54)/(1-J54)-1</f>
+        <v/>
+      </c>
+      <c r="L58" s="68">
+        <f>(1+L50)*(1-L54)/(1-K54)-1</f>
+        <v/>
+      </c>
+      <c r="M58" s="68">
+        <f>(1+M50)*(1-M54)/(1-L54)-1</f>
+        <v/>
+      </c>
+      <c r="N58" s="68">
+        <f>(1+N50)*(1-N54)/(1-M54)-1</f>
+        <v/>
+      </c>
+      <c r="O58" s="68">
+        <f>(1+O50)*(1-O54)/(1-N54)-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="14.4" customHeight="1"/>
+    <row r="60" ht="14.4" customHeight="1">
+      <c r="B60" s="69" t="inlineStr">
         <is>
           <t>▸ DETAIL: subject rent source by year &amp; reconciliation (grouped — click − to collapse)</t>
         </is>
       </c>
     </row>
-    <row r="52" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B52" s="60" t="inlineStr">
+    <row r="61" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B61" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y6  Q3 2019–Q2 2020</t>
         </is>
       </c>
-      <c r="E52" s="60" t="inlineStr">
+      <c r="E61" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="53" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B53" s="60" t="inlineStr">
+    <row r="62" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B62" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y5  Q3 2020–Q2 2021</t>
         </is>
       </c>
-      <c r="E53" s="60" t="inlineStr">
+      <c r="E62" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="54" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B54" s="60" t="inlineStr">
+    <row r="63" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B63" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y4  Q3 2021–Q2 2022</t>
         </is>
       </c>
-      <c r="E54" s="60" t="inlineStr">
+      <c r="E63" s="71" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="55" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B55" s="60" t="inlineStr">
+    <row r="64" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B64" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y3  Q3 2022–Q2 2023</t>
         </is>
       </c>
-      <c r="E55" s="60" t="inlineStr">
+      <c r="E64" s="71" t="inlineStr">
         <is>
           <t>RealPage</t>
         </is>
       </c>
     </row>
-    <row r="56" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B56" s="60" t="inlineStr">
+    <row r="65" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B65" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y2  Q3 2023–Q2 2024</t>
         </is>
       </c>
-      <c r="E56" s="60" t="inlineStr">
+      <c r="E65" s="71" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
-    <row r="57" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B57" s="60" t="inlineStr">
+    <row r="66" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B66" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  -Y1  Q3 2024–Q2 2025</t>
         </is>
       </c>
-      <c r="E57" s="60" t="inlineStr">
+      <c r="E66" s="71" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
-    <row r="58" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B58" s="60" t="inlineStr">
+    <row r="67" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B67" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  Y0  Q3 2025–Q2 2026</t>
         </is>
       </c>
-      <c r="E58" s="60" t="inlineStr">
+      <c r="E67" s="71" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
     </row>
-    <row r="59" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B59" s="60" t="inlineStr">
+    <row r="68" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B68" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  UC scheduled vs CoStar UC</t>
         </is>
       </c>
-      <c r="E59" s="60" t="inlineStr">
+      <c r="E68" s="71" t="inlineStr">
         <is>
           <t>885 / 336</t>
         </is>
       </c>
     </row>
-    <row r="60" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
-      <c r="B60" s="29" t="inlineStr">
+    <row r="69" hidden="1" outlineLevel="1" ht="14.4" customHeight="1">
+      <c r="B69" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  As-of 2026 Q2 QTD is partial (QTD); occupancy is point-in-time, Y0 flow sums partial.</t>
         </is>
       </c>
     </row>
-    <row r="61" ht="14.4" customHeight="1"/>
-    <row r="62" ht="14.4" customHeight="1"/>
+    <row r="70" ht="14.4" customHeight="1"/>
+    <row r="71" ht="14.4" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B2:O2"/>
@@ -3237,62 +3594,62 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="61" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>Property</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr">
+      <c r="B1" s="57" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="C1" s="61" t="inlineStr">
+      <c r="C1" s="57" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="D1" s="61" t="inlineStr">
+      <c r="D1" s="57" t="inlineStr">
         <is>
           <t>Year Built</t>
         </is>
       </c>
-      <c r="E1" s="61" t="inlineStr">
+      <c r="E1" s="57" t="inlineStr">
         <is>
           <t>Est. Delivery</t>
         </is>
       </c>
-      <c r="F1" s="61" t="inlineStr">
+      <c r="F1" s="57" t="inlineStr">
         <is>
           <t>Bucket</t>
         </is>
       </c>
-      <c r="G1" s="61" t="inlineStr">
+      <c r="G1" s="57" t="inlineStr">
         <is>
           <t>CoStar Occ</t>
         </is>
       </c>
-      <c r="H1" s="61" t="inlineStr">
+      <c r="H1" s="57" t="inlineStr">
         <is>
           <t>RealPage Occ</t>
         </is>
       </c>
-      <c r="I1" s="61" t="inlineStr">
+      <c r="I1" s="57" t="inlineStr">
         <is>
           <t>CoStar Ask Rent</t>
         </is>
       </c>
-      <c r="J1" s="61" t="inlineStr">
+      <c r="J1" s="57" t="inlineStr">
         <is>
           <t>RealPage Eff Rent</t>
         </is>
       </c>
-      <c r="K1" s="61" t="inlineStr">
+      <c r="K1" s="57" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="L1" s="61" t="inlineStr">
+      <c r="L1" s="57" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3325,16 +3682,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G2" s="62" t="n">
+      <c r="G2" s="72" t="n">
         <v>0.926316</v>
       </c>
-      <c r="H2" s="62" t="n">
+      <c r="H2" s="72" t="n">
         <v>0.953</v>
       </c>
-      <c r="I2" s="63" t="n">
+      <c r="I2" s="73" t="n">
         <v>1795</v>
       </c>
-      <c r="J2" s="63" t="n">
+      <c r="J2" s="73" t="n">
         <v>1709</v>
       </c>
       <c r="K2" t="inlineStr">
@@ -3375,16 +3732,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G3" s="62" t="n">
+      <c r="G3" s="72" t="n">
         <v>0.902778</v>
       </c>
-      <c r="H3" s="62" t="n">
+      <c r="H3" s="72" t="n">
         <v>0.95</v>
       </c>
-      <c r="I3" s="63" t="n">
+      <c r="I3" s="73" t="n">
         <v>1765</v>
       </c>
-      <c r="J3" s="63" t="n">
+      <c r="J3" s="73" t="n">
         <v>1793</v>
       </c>
       <c r="K3" t="inlineStr">
@@ -3425,16 +3782,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G4" s="62" t="n">
+      <c r="G4" s="72" t="n">
         <v>0.879365</v>
       </c>
-      <c r="H4" s="62" t="n">
+      <c r="H4" s="72" t="n">
         <v>0.911</v>
       </c>
-      <c r="I4" s="63" t="n">
+      <c r="I4" s="73" t="n">
         <v>1836</v>
       </c>
-      <c r="J4" s="63" t="n">
+      <c r="J4" s="73" t="n">
         <v>1821</v>
       </c>
       <c r="K4" t="inlineStr">
@@ -3475,16 +3832,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G5" s="62" t="n">
+      <c r="G5" s="72" t="n">
         <v>0.92</v>
       </c>
-      <c r="H5" s="62" t="n">
+      <c r="H5" s="72" t="n">
         <v>0.929</v>
       </c>
-      <c r="I5" s="63" t="n">
+      <c r="I5" s="73" t="n">
         <v>1861</v>
       </c>
-      <c r="J5" s="63" t="n">
+      <c r="J5" s="73" t="n">
         <v>1439</v>
       </c>
       <c r="K5" t="inlineStr">
@@ -3525,16 +3882,16 @@
           <t>STABILIZED / STABILIZING</t>
         </is>
       </c>
-      <c r="G6" s="62" t="n">
+      <c r="G6" s="72" t="n">
         <v>0.948454</v>
       </c>
-      <c r="H6" s="62" t="n">
+      <c r="H6" s="72" t="n">
         <v>0.952</v>
       </c>
-      <c r="I6" s="63" t="n">
+      <c r="I6" s="73" t="n">
         <v>1897</v>
       </c>
-      <c r="J6" s="63" t="n">
+      <c r="J6" s="73" t="n">
         <v>1927</v>
       </c>
       <c r="K6" t="inlineStr">
@@ -3571,10 +3928,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G7" s="62" t="n"/>
-      <c r="H7" s="62" t="n"/>
-      <c r="I7" s="63" t="n"/>
-      <c r="J7" s="63" t="n"/>
+      <c r="G7" s="72" t="n"/>
+      <c r="H7" s="72" t="n"/>
+      <c r="I7" s="73" t="n"/>
+      <c r="J7" s="73" t="n"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3613,10 +3970,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G8" s="62" t="n"/>
-      <c r="H8" s="62" t="n"/>
-      <c r="I8" s="63" t="n"/>
-      <c r="J8" s="63" t="n"/>
+      <c r="G8" s="72" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="73" t="n"/>
+      <c r="J8" s="73" t="n"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3655,10 +4012,10 @@
           <t>UNDER CONSTRUCTION</t>
         </is>
       </c>
-      <c r="G9" s="62" t="n"/>
-      <c r="H9" s="62" t="n"/>
-      <c r="I9" s="63" t="n"/>
-      <c r="J9" s="63" t="n"/>
+      <c r="G9" s="72" t="n"/>
+      <c r="H9" s="72" t="n"/>
+      <c r="I9" s="73" t="n"/>
+      <c r="J9" s="73" t="n"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3697,10 +4054,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G10" s="62" t="n"/>
-      <c r="H10" s="62" t="n"/>
-      <c r="I10" s="63" t="n"/>
-      <c r="J10" s="63" t="n"/>
+      <c r="G10" s="72" t="n"/>
+      <c r="H10" s="72" t="n"/>
+      <c r="I10" s="73" t="n"/>
+      <c r="J10" s="73" t="n"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3739,10 +4096,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G11" s="62" t="n"/>
-      <c r="H11" s="62" t="n"/>
-      <c r="I11" s="63" t="n"/>
-      <c r="J11" s="63" t="n"/>
+      <c r="G11" s="72" t="n"/>
+      <c r="H11" s="72" t="n"/>
+      <c r="I11" s="73" t="n"/>
+      <c r="J11" s="73" t="n"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>CoStar+RealPage</t>
@@ -3781,10 +4138,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G12" s="62" t="n"/>
-      <c r="H12" s="62" t="n"/>
-      <c r="I12" s="63" t="n"/>
-      <c r="J12" s="63" t="n"/>
+      <c r="G12" s="72" t="n"/>
+      <c r="H12" s="72" t="n"/>
+      <c r="I12" s="73" t="n"/>
+      <c r="J12" s="73" t="n"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3815,10 +4172,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G13" s="62" t="n"/>
-      <c r="H13" s="62" t="n"/>
-      <c r="I13" s="63" t="n"/>
-      <c r="J13" s="63" t="n"/>
+      <c r="G13" s="72" t="n"/>
+      <c r="H13" s="72" t="n"/>
+      <c r="I13" s="73" t="n"/>
+      <c r="J13" s="73" t="n"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3849,10 +4206,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G14" s="62" t="n"/>
-      <c r="H14" s="62" t="n"/>
-      <c r="I14" s="63" t="n"/>
-      <c r="J14" s="63" t="n"/>
+      <c r="G14" s="72" t="n"/>
+      <c r="H14" s="72" t="n"/>
+      <c r="I14" s="73" t="n"/>
+      <c r="J14" s="73" t="n"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3883,10 +4240,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G15" s="62" t="n"/>
-      <c r="H15" s="62" t="n"/>
-      <c r="I15" s="63" t="n"/>
-      <c r="J15" s="63" t="n"/>
+      <c r="G15" s="72" t="n"/>
+      <c r="H15" s="72" t="n"/>
+      <c r="I15" s="73" t="n"/>
+      <c r="J15" s="73" t="n"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3917,10 +4274,10 @@
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="G16" s="62" t="n"/>
-      <c r="H16" s="62" t="n"/>
-      <c r="I16" s="63" t="n"/>
-      <c r="J16" s="63" t="n"/>
+      <c r="G16" s="72" t="n"/>
+      <c r="H16" s="72" t="n"/>
+      <c r="I16" s="73" t="n"/>
+      <c r="J16" s="73" t="n"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>RealPage</t>
@@ -3957,7 +4314,7 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="64" t="inlineStr">
+      <c r="B2" s="74" t="inlineStr">
         <is>
           <t>PIPELINE DILIGENCE</t>
         </is>
@@ -4006,12 +4363,12 @@
           <t>Riverview at Clear Creek</t>
         </is>
       </c>
-      <c r="C4" s="65" t="inlineStr">
+      <c r="C4" s="75" t="inlineStr">
         <is>
           <t>298</t>
         </is>
       </c>
-      <c r="D4" s="65" t="n"/>
+      <c r="D4" s="75" t="n"/>
       <c r="E4" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4035,12 +4392,12 @@
           <t>Lenox Clear Creek</t>
         </is>
       </c>
-      <c r="C5" s="65" t="inlineStr">
+      <c r="C5" s="75" t="inlineStr">
         <is>
           <t>336</t>
         </is>
       </c>
-      <c r="D5" s="65" t="inlineStr">
+      <c r="D5" s="75" t="inlineStr">
         <is>
           <t>Q3 2027</t>
         </is>
@@ -4068,12 +4425,12 @@
           <t>Dakota at Kemah</t>
         </is>
       </c>
-      <c r="C6" s="65" t="inlineStr">
+      <c r="C6" s="75" t="inlineStr">
         <is>
           <t>229</t>
         </is>
       </c>
-      <c r="D6" s="65" t="inlineStr">
+      <c r="D6" s="75" t="inlineStr">
         <is>
           <t>Q1 2027</t>
         </is>
@@ -4101,12 +4458,12 @@
           <t>The League I</t>
         </is>
       </c>
-      <c r="C7" s="65" t="inlineStr">
+      <c r="C7" s="75" t="inlineStr">
         <is>
           <t>304</t>
         </is>
       </c>
-      <c r="D7" s="65" t="inlineStr">
+      <c r="D7" s="75" t="inlineStr">
         <is>
           <t>Q3 2026</t>
         </is>
@@ -4134,12 +4491,12 @@
           <t>The Edge at Seabrook Town Centre</t>
         </is>
       </c>
-      <c r="C8" s="65" t="inlineStr">
+      <c r="C8" s="75" t="inlineStr">
         <is>
           <t>320</t>
         </is>
       </c>
-      <c r="D8" s="65" t="inlineStr">
+      <c r="D8" s="75" t="inlineStr">
         <is>
           <t>Q2 2028</t>
         </is>
@@ -4167,12 +4524,12 @@
           <t>The League Future Phases</t>
         </is>
       </c>
-      <c r="C9" s="65" t="inlineStr">
+      <c r="C9" s="75" t="inlineStr">
         <is>
           <t>400</t>
         </is>
       </c>
-      <c r="D9" s="65" t="n"/>
+      <c r="D9" s="75" t="n"/>
       <c r="E9" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4196,12 +4553,12 @@
           <t>Residences at Highland Center</t>
         </is>
       </c>
-      <c r="C10" s="65" t="inlineStr">
+      <c r="C10" s="75" t="inlineStr">
         <is>
           <t>275</t>
         </is>
       </c>
-      <c r="D10" s="65" t="n"/>
+      <c r="D10" s="75" t="n"/>
       <c r="E10" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4225,12 +4582,12 @@
           <t>Seabrook Plaza</t>
         </is>
       </c>
-      <c r="C11" s="65" t="inlineStr">
+      <c r="C11" s="75" t="inlineStr">
         <is>
           <t>260</t>
         </is>
       </c>
-      <c r="D11" s="65" t="n"/>
+      <c r="D11" s="75" t="n"/>
       <c r="E11" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4254,12 +4611,12 @@
           <t>Avalon at Kemah I</t>
         </is>
       </c>
-      <c r="C12" s="65" t="inlineStr">
+      <c r="C12" s="75" t="inlineStr">
         <is>
           <t>198</t>
         </is>
       </c>
-      <c r="D12" s="65" t="n"/>
+      <c r="D12" s="75" t="n"/>
       <c r="E12" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4283,12 +4640,12 @@
           <t>Avalon at Kemah II</t>
         </is>
       </c>
-      <c r="C13" s="65" t="inlineStr">
+      <c r="C13" s="75" t="inlineStr">
         <is>
           <t>228</t>
         </is>
       </c>
-      <c r="D13" s="65" t="n"/>
+      <c r="D13" s="75" t="n"/>
       <c r="E13" s="35" t="inlineStr">
         <is>
           <t>proposed</t>
@@ -4307,7 +4664,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="64" t="inlineStr">
+      <c r="B15" s="74" t="inlineStr">
         <is>
           <t>SHADOW SUPPLY (latent / untracked — watch list)</t>
         </is>
@@ -4356,8 +4713,8 @@
           <t>Westland Ranch MPC potential MF tract</t>
         </is>
       </c>
-      <c r="C17" s="65" t="n"/>
-      <c r="D17" s="65" t="n"/>
+      <c r="C17" s="75" t="n"/>
+      <c r="D17" s="75" t="n"/>
       <c r="E17" s="35" t="inlineStr">
         <is>
           <t>planned/speculative</t>
@@ -4381,8 +4738,8 @@
           <t>FM-518 / Main St corridor mixed-use capacity</t>
         </is>
       </c>
-      <c r="C18" s="65" t="n"/>
-      <c r="D18" s="65" t="n"/>
+      <c r="C18" s="75" t="n"/>
+      <c r="D18" s="75" t="n"/>
       <c r="E18" s="35" t="inlineStr">
         <is>
           <t>zoning/entitlement capacity</t>
@@ -4406,8 +4763,8 @@
           <t>Webster / SH-3 &amp; Bay Area Blvd MF node</t>
         </is>
       </c>
-      <c r="C19" s="65" t="n"/>
-      <c r="D19" s="65" t="n"/>
+      <c r="C19" s="75" t="n"/>
+      <c r="D19" s="75" t="n"/>
       <c r="E19" s="35" t="inlineStr">
         <is>
           <t>redevelopment node</t>
@@ -4431,8 +4788,8 @@
           <t>Friendswood multifamily</t>
         </is>
       </c>
-      <c r="C20" s="65" t="n"/>
-      <c r="D20" s="65" t="n"/>
+      <c r="C20" s="75" t="n"/>
+      <c r="D20" s="75" t="n"/>
       <c r="E20" s="35" t="inlineStr">
         <is>
           <t>none confirmed</t>

</xml_diff>